<commit_message>
está com 2 comprimento por isso erros na coluna
</commit_message>
<xml_diff>
--- a/NomeEletrica.xlsx
+++ b/NomeEletrica.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1113" uniqueCount="668">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1332" uniqueCount="540">
   <si>
     <t>Descricao_Limpa</t>
   </si>
@@ -1165,859 +1165,475 @@
     <t>LS</t>
   </si>
   <si>
-    <t>HIDROLETE CONDUITE B 3/4 AMARELO 50M HIDROLET 0.024 3/4" 1.0 AMARELO HIDROLETE 432</t>
-  </si>
-  <si>
-    <t>CORRUTECH CONDUITE A 1/2 CINZA REF 50M 0.024 1/2" 1.0 CINZA CORRUTECH 433</t>
-  </si>
-  <si>
-    <t>TRAMONTINA CAIXA LUZ 4X2 AMARELO 0.024 1.0 4x2 AMARELO TRAMONTINA 434</t>
-  </si>
-  <si>
-    <t>TRAMONTINA ELE CANALETA 20X10X2M BRANCO S/DIV FIT 0.024 1.0 BRANCO TRAMONTINA ELE 435</t>
-  </si>
-  <si>
-    <t>STECK DISJUNTOR DIN UNIPOLAR 10A CURVA C 0.024 10.0A 1P 8.0 STECK 436</t>
-  </si>
-  <si>
-    <t>STECK DISJUNTOR DIN BIPOLAR 40A CURVA C 0.024 40.0A 2P 8.0 STECK 436</t>
-  </si>
-  <si>
-    <t>STECK DISJUNTOR DIN BIPOLAR 50A CURVA C 0.024 50.0A 2P 8.0 STECK 436</t>
-  </si>
-  <si>
-    <t>FC CAIXINHA LUZ PVC 4X4 AMARELO 0.031 11.0 4x4 AMARELO FC 437</t>
-  </si>
-  <si>
-    <t>KRONA LUVA CORRUGADO C 25MM 3/4 0.048 25mm 3.0 KRONA 438</t>
-  </si>
-  <si>
-    <t>THOMPSON PLAFONIER RED PVC SOQ PORCELANA BRANCO 0.032 14.0 BRANCO THOMPSON 439</t>
-  </si>
-  <si>
-    <t>THOMPSON LAMPADA BOLINHA 15X127 SORT 0.024 4.5 THOMPSON 440</t>
-  </si>
-  <si>
-    <t>FOXLUX REFLETOR LED 30W ALUMINIO 6500K 0.024 19.0 FOXLUX 441</t>
-  </si>
-  <si>
-    <t>FOXLUX LAMPADA LED TUBULAR T8 18W1850LM 6500K 0.024 3.0 FOXLUX 442</t>
-  </si>
-  <si>
-    <t>INJEREST CAIXINHA LUZ PE 4X2 PRETO 0.031 5.0 4x2 PRETO INJEREST 443</t>
-  </si>
-  <si>
-    <t>HIDROLETE CONDUITE A 1/2 AMARELO 50M HIDROLET 0.024 1/2" 1.0 AMARELO HIDROLETE 432</t>
-  </si>
-  <si>
-    <t>LUKMA DISJUNTOR DIN BIPOLAR 50A CURVA C 0.024 50.0A 2P 25.0 LUKMA 444</t>
-  </si>
-  <si>
-    <t>CONDUITE B 3/4 CINZA REF 50M CORRUTECH 0.024 3/4" 1.0 CINZA CORRUTECH 433</t>
-  </si>
-  <si>
-    <t>THOMPSON RECEPTACULO E27 1451 0.024 5.0 THOMPSON 445</t>
-  </si>
-  <si>
-    <t>SUBRAP SUPORTE DISJUNTOR DIN BAIXO DESTACAVEL 20 UND 0.048 3.5 SUBRAP 446</t>
-  </si>
-  <si>
-    <t>SCHNEIDER BARRAMENTO DIN 1P 80A 12 POLOS EZ9X33112 0.048 1P 3.0 SCHNEIDER 447</t>
-  </si>
-  <si>
-    <t>SCHNEIDER BARRAMENTO DIN 2P 80A 12 POLOS EZ9X33212 0.048 2P 3.0 SCHNEIDER 447</t>
-  </si>
-  <si>
-    <t>BARRAMENTO NEU/TERR 08 T COMSUP EZ9E33B08 0.048 GENÉRICO 448</t>
-  </si>
-  <si>
-    <t>CONECTOR WAGO 3P 08 A 4,0M 32A 0.024 32.0A 3P WAGO 449</t>
-  </si>
-  <si>
-    <t>CONECTOR WAGO 2P 08 A 4,0M 32A 0.024 32.0A 2P WAGO 449</t>
-  </si>
-  <si>
-    <t>CORRUTECH CONDUITE C 1,0 CINZA 25M 0.024 1" 1.0 CINZA CORRUTECH 433</t>
-  </si>
-  <si>
-    <t>CONDUITE B 3/4 CINZA 50M CORRUTECH 0.024 3/4" 1.0 CINZA CORRUTECH 433</t>
-  </si>
-  <si>
-    <t>CONECTOR PORCELANA 6MM 3P COM100 BRASFORT 0.024 3P 6mm 1.0 BRASFORT 450</t>
-  </si>
-  <si>
-    <t>CONECTOR PORCELANA 16MM 3P COM12 BRASFORT 0.024 3P 16mm 1.0 BRASFORT 450</t>
-  </si>
-  <si>
-    <t>STECK DISJUNTOR DIN UNIPOLAR 20A CURVA C 0.024 20.0A 1P 8.0 STECK 436</t>
-  </si>
-  <si>
-    <t>SISTEMA ILUMI BRANCO CANAL20X10X2M ADE/DI 0.024 200.0 BRANCO ILUMI 451</t>
-  </si>
-  <si>
-    <t>ILUMI SOQUETE SEM CHAVE NYLON 0.024 3.0 ILUMI 452</t>
-  </si>
-  <si>
-    <t>THOMPSON CONECTOR 03 BORNE 10MM 0.031 10mm 20.0 THOMPSON 453</t>
-  </si>
-  <si>
-    <t>THOMPSON CONECTOR 03 BORNE 16MM 0.031 16mm 2.5 THOMPSON 453</t>
-  </si>
-  <si>
-    <t>SISTEMA STECK CANALETA BRANCO 20X10X2M ADES 0.024 0.39 BRANCO STECK 454</t>
-  </si>
-  <si>
-    <t>PINO PORTA LAMPADA ADAPTADOR PERLEX SEGURANÇA 122 0.024 PERLEX 455</t>
-  </si>
-  <si>
-    <t>TRAMONTINA CAIXINHA LUZ PVC 4X2 AMARELO /044 0.031 5.0 4x2 AMARELO TRAMONTINA 434</t>
-  </si>
-  <si>
-    <t>TRAMONTINA CORRUGADO PVC 25MM AMARELO METRO/50 0.024 25mm 50.0 AMARELO TRAMONTINA 456</t>
-  </si>
-  <si>
-    <t>TRAMONTINA CAIXINHA LUZ DRYWALL 4X2 AMARELO /071 0.031 5.0 4x2 AMARELO TRAMONTINA 434</t>
-  </si>
-  <si>
-    <t>CAIXINHA LUZ AMARELA TRAMONTINA 4X4 0.031 4x4 GENÉRICO 434</t>
-  </si>
-  <si>
-    <t>TRAMONTINA CAIXINHA LUZ PVC 3X3 AMARELO /043 0.031 9.0 3x3 AMARELO TRAMONTINA 434</t>
-  </si>
-  <si>
-    <t>TRAMONTINA CORRUGADO PVC 32MM AMARELO METRO/25 0.024 32mm 3.0 AMARELO TRAMONTINA 456</t>
-  </si>
-  <si>
-    <t>INTERNEED PLAFONIER RED PVC SOQ PORCELANA BRANCO 0.032 14.5 BRANCO INTERNEED 439</t>
-  </si>
-  <si>
-    <t>CONECTOR INTERNEED PORCELANA 10MM TRIF 0.024 10mm GENÉRICO 457</t>
-  </si>
-  <si>
-    <t>PASSA FIO TOR ALF 15MT 0.024 GENÉRICO 458</t>
-  </si>
-  <si>
-    <t>STECK BARRAMENTO DIN 2P 80A 12 POLOS 2F210B 0.048 2P 3.0 STECK 459</t>
-  </si>
-  <si>
-    <t>CENTRI STECK PVC 04 DISJUNTOR DIN SOB BRANCO SCT4 0.048 04 BRANCO GENÉRICO 460</t>
-  </si>
-  <si>
-    <t>CENTRI STECK PVC 02 DISJUNTOR DIN SOB BRANCO SCT2 0.048 02 BRANCO GENÉRICO 460</t>
-  </si>
-  <si>
-    <t>CENTRI STECK PVC 12 DISJUNTOR DIN EMBALAGEM BRANCO 0.048 12 BRANCO GENÉRICO 460</t>
-  </si>
-  <si>
-    <t>STECK CENTRO DISTRIBUIÇÃO DISJUNTOR DIN 08 EMBALAGEM BRANCO 1P 0.024 1P 23.0 08 BRANCO STECK 461</t>
-  </si>
-  <si>
-    <t>DISJUNTOR STECK SERIE SD61 16A 1P CURVA C 3KA 0.024 16.0A 1P GENÉRICO 462</t>
-  </si>
-  <si>
-    <t>DISJUNTOR STECK SERIE SD61 20A 1P CURVA C 3KA 0.024 20.0A 1P GENÉRICO 462</t>
-  </si>
-  <si>
-    <t>STECK DISJUNTOR DIN UNIPOLAR 25A CURVA C 0.024 25.0A 1P 8.0 STECK 436</t>
-  </si>
-  <si>
-    <t>STECK DISJUNTOR DIN UNIPOLAR 32A CURVA C 0.024 32.0A 1P 8.0 STECK 436</t>
-  </si>
-  <si>
-    <t>DISJUNTOR STECK SERIE SD61 40A 1P CURVA C 3KA 0.024 40.0A 1P GENÉRICO 462</t>
-  </si>
-  <si>
-    <t>STECK DISJUNTOR DIN BIPOLAR 10A CURVA C 0.024 10.0A 2P 8.0 STECK 436</t>
-  </si>
-  <si>
-    <t>STECK DISJUNTOR DIN BIPOLAR 32A CURVA C 0.024 32.0A 2P 8.0 STECK 436</t>
-  </si>
-  <si>
-    <t>DISJUNTOR STECK SERIE SD62 40A 2P CURVA C 3KA 0.024 40.0A 2P GENÉRICO 462</t>
-  </si>
-  <si>
-    <t>DISJUNTOR STECK SERIE SD62 50A 2P CURVA C 3KA 0.024 50.0A 2P GENÉRICO 462</t>
-  </si>
-  <si>
-    <t>STECK DISJUNTOR DIN BIPOLAR 63A CURVA C 0.024 63.0A 2P 8.0 STECK 436</t>
-  </si>
-  <si>
-    <t>SISTEMA X STECK CANALETA BRANCO COMFITA 20X2MT 0.024 BRANCO GENÉRICO 454</t>
-  </si>
-  <si>
-    <t>JOGO SOQUETE EDA ENCAIXE 1/43/8 40PC 0.024 1" GENÉRICO 463</t>
-  </si>
-  <si>
-    <t>SISTEMA FAME CANALETA BRANCO 20X10X2M ADES 0.024 200.0 BRANCO FAME 454</t>
-  </si>
-  <si>
-    <t>SISTEMA X ALUMBRA CANALETA BRANCO COMFITA 20X2MT 0.024 BRANCO ALUMBRA 464</t>
-  </si>
-  <si>
-    <t>SISTEMA X ALUMBRA CANALETA BRANCO COMFITA 10X2MT 0.024 BRANCO ALUMBRA 464</t>
-  </si>
-  <si>
-    <t>BIKI CENTRO DISTRIBUIÇÃO DISJUNTOR DIN/NEMA 03/04 EMBALAGEM BRANCO 0.024 14.0 03 BRANCO BIKI 461</t>
-  </si>
-  <si>
-    <t>FC PLAFONIER RED PVC SOQ PORCELANA BRANCO 0.032 15.0 BRANCO FC 439</t>
-  </si>
-  <si>
-    <t>FC PLAFONIER RED PVC SOQ PORCELANA PRETO 0.032 14.5 PRETO FC 439</t>
-  </si>
-  <si>
-    <t>FC CAIXINHA LUZ PVC 4X2 AMARELO 0.031 7.0 4x2 AMARELO FC 437</t>
-  </si>
-  <si>
-    <t>FC PASSA FIO 10M ALMA ACO 0.024 16.5 FC 465</t>
-  </si>
-  <si>
-    <t>SIL CABO FLEXIVEL 1,50 PRETO R/100M 0.008 1" 22.0 PRETO SIL 466</t>
-  </si>
-  <si>
-    <t>CABO FLEXÍVEL 6,00MM X 100M AZUL 0.008 6.00mm AZUL GENÉRICO 467</t>
-  </si>
-  <si>
-    <t>CABO FLEXÍVEL 6,00MM X 100M PRETO 0.008 6.00mm PRETO GENÉRICO 467</t>
-  </si>
-  <si>
-    <t>CABO FLEXÍVEL 6,00MM X 100M VERMELHO 0.008 6.00mm VERMELHO GENÉRICO 467</t>
-  </si>
-  <si>
-    <t>CABO FLEXÍVEL PARALELO 2 X 1,5MM X 100M BRANCO 0.008 1.5mm BRANCO GENÉRICO 468</t>
-  </si>
-  <si>
-    <t>SIL CABO FLEXIVEL 1,50 AMARELO R/100M 0.008 1" 23.0 AMARELO SIL 466</t>
-  </si>
-  <si>
-    <t>SENSOR PRESENÇA EXATRON COMSOQ E27 XC BIVOLT 0.007 GENÉRICO 469</t>
-  </si>
-  <si>
-    <t>CONDUITE CORRUGADO AMARELO D 1 R/50 0.048 1" AMARELO GENÉRICO 470</t>
-  </si>
-  <si>
-    <t>CONDUITE CORRUGADO AMARELO C 3/4 R/50 0.048 3/4" AMARELO GENÉRICO 470</t>
-  </si>
-  <si>
-    <t>CONDUITE CORRUGADO AMARELO B 5/8 R/50 0.048 5/8" AMARELO GENÉRICO 470</t>
-  </si>
-  <si>
-    <t>CONDUITE CORRUGADO AMARELO A 1/2 R/100 0.048 1/2" AMARELO GENÉRICO 470</t>
-  </si>
-  <si>
-    <t>CONDUITE CORRUGADO PRETO D 1 R/50 0.048 1" PRETO GENÉRICO 470</t>
-  </si>
-  <si>
-    <t>CONDUITE CORRUGADO PRETO C 3/4 RL/50 0.048 3/4" PRETO GENÉRICO 471</t>
-  </si>
-  <si>
-    <t>CONDUITE CORRUGADO PRETO A 1/2 RL/100 0.048 1/2" PRETO GENÉRICO 470</t>
-  </si>
-  <si>
-    <t>PASSA FIO PROAQUA SUPER COMALMA DE ACO10M 0.024 PROAQUA 472</t>
-  </si>
-  <si>
-    <t>PASSA FIO PROAQUA SUPER COMALMA DE ACO15M 0.024 PROAQUA 472</t>
-  </si>
-  <si>
-    <t>PASSA FIO PROAQUA SUPER COMALMA DE ACO20M 0.024 PROAQUA 472</t>
-  </si>
-  <si>
-    <t>PASSA FIO PROAQUA SUPER COMALMA DE ACO30M 0.024 PROAQUA 472</t>
-  </si>
-  <si>
-    <t>PENZEL TERM PREISOL PINO AZUL 1,5MM/2,5MM C9MM 0.024 1.5mm 1.5 AZUL PENZEL 473</t>
-  </si>
-  <si>
-    <t>PENZEL TERM PREISOL PINO AMARELO 4MM/6,00MM C13MM 0.024 4mm 1.0 AMARELO PENZEL 473</t>
-  </si>
-  <si>
-    <t>PENZEL TERM PREISOL ANEL F4 VERMELHO 0,5MM/1,5MM 0.024 0.5mm 11.5 VERMELHO PENZEL 474</t>
-  </si>
-  <si>
-    <t>PENZEL TERM PREISOL ANEL F4 AZUL 1,5MM/2,5MM 0.024 1.5mm 11.5 AZUL PENZEL 473</t>
-  </si>
-  <si>
-    <t>AMANCO CURVA ELETRODUTO H 11/4X90 0.024 24.0 AMANCO 475</t>
-  </si>
-  <si>
-    <t>AMANCO CURVA ELETRODUTO F 11/2X90 0.024 24.0 AMANCO 475</t>
-  </si>
-  <si>
-    <t>RECEPTACULO CANIELLO LATAO 1451 0.024 GENÉRICO 476</t>
-  </si>
-  <si>
-    <t>PINO PORTA LAMPADA THOMPSON PRETO 1423 0.024 PRETO GENÉRICO 477</t>
-  </si>
-  <si>
-    <t>THOMPSOM LAMPADA GELAD/MICROONDAS E14 15W 127V 0.024 THOMPSOM 478</t>
-  </si>
-  <si>
-    <t>THOMPSON CENTRO DISTRIBUIÇÃO DISJUNTOR DIN/NEMA 06/08 EMBALAGEM CINZA 0.024 25.0 08 CINZA THOMPSON 479</t>
-  </si>
-  <si>
-    <t>THOMPSOM CENTRI PVC 12/16 DISJUNTOR BRANCO/FUME EMBALAGEM 0.048 12 BRANCO THOMPSOM 480</t>
-  </si>
-  <si>
-    <t>THOMPSOM CENTRI PVC 06/08 DISJUNTOR BRANCO EMBALAGEM 0.048 08 BRANCO THOMPSOM 480</t>
-  </si>
-  <si>
-    <t>THOMPSOM CENTRI PVC 12/16 DISJUNTOR BRANCO EMBALAGEM 0.048 12 BRANCO THOMPSOM 480</t>
-  </si>
-  <si>
-    <t>FOXLUX RECEPTACULO E27 1451 FX09 0.024 4.0 FOXLUX 445</t>
-  </si>
-  <si>
-    <t>FOXLUX SOQUETE C/ PLUG E27 PRETO 0.024 4.0 PRETO FOXLUX 481</t>
-  </si>
-  <si>
-    <t>FOXLUX FILTRO ADSL 2 SAIDAS 0.008 13.0 FOXLUX 482</t>
-  </si>
-  <si>
-    <t>SOQUETE COMRABICHO RADIAL LATAO 0.024 RADIAL 483</t>
-  </si>
-  <si>
-    <t>PINO PORTA LAMPADA ADAPTADOR RADIAL PRETO 113 0.024 PRETO RADIAL 455</t>
-  </si>
-  <si>
-    <t>QUALITRONIX SOQUETE SENSOR PRESENCA E27 COMFTC BRANCO 0.048 11.0 BRANCO QUALITRONIX 484</t>
-  </si>
-  <si>
-    <t>TOMADINHA COMRABICHO REDY 107 0.007 REDY 485</t>
-  </si>
-  <si>
-    <t>PLAFON DECORA PVC REDY BRANCO 0.024 BRANCO REDY 486</t>
-  </si>
-  <si>
-    <t>SOQUETE COMRABICHO REDY 102 0.024 REDY 483</t>
-  </si>
-  <si>
-    <t>FIO CABO AUTO COBRECOM 1,50 AMARELO 0.024 1" AMARELO COBRECOM 487</t>
-  </si>
-  <si>
-    <t>FIO CABO AUTO COBRECOM 1,50 BRANCO 0.024 1" BRANCO COBRECOM 487</t>
-  </si>
-  <si>
-    <t>FIO CABO AUTO COBRECOM 1,50 VERMELHO 0.024 1" VERMELHO COBRECOM 487</t>
-  </si>
-  <si>
-    <t>FIO CABO AUTO COBRECOM 1,50 PRETO 0.024 1" PRETO COBRECOM 487</t>
-  </si>
-  <si>
-    <t>FIO CABO AUTO COBRECOM 6,00 AZUL 0.024 AZUL COBRECOM 487</t>
-  </si>
-  <si>
-    <t>FIO CABO AUTO COBRECOM 6,00 VERMELHO 0.024 VERMELHO COBRECOM 487</t>
-  </si>
-  <si>
-    <t>FIO CABO AUTO COBRECOM 6,00 PRETO 0.024 PRETO COBRECOM 487</t>
-  </si>
-  <si>
-    <t>FIO CABO AUTO COBRECOM 10,00 AZUL 0.024 AZUL COBRECOM 487</t>
-  </si>
-  <si>
-    <t>FIO CABO AUTO COBRECOM 10,00 PRETO 0.024 PRETO COBRECOM 487</t>
-  </si>
-  <si>
-    <t>INTERFONE HDL PORT ELETRICA F8SN 0.024 GENÉRICO 488</t>
-  </si>
-  <si>
-    <t>CENTRI ILUMI PVC 12/16 DISJUNTOR BRANCO EMBALAGEM 0.048 12 BRANCO ILUMI 480</t>
-  </si>
-  <si>
-    <t>ILUMI SOQUETE COMRABICHO E27 NYLON 0.024 3.0 ILUMI 489</t>
-  </si>
-  <si>
-    <t>LAMPADA LED A60 09W860LM 6500K 0.024 GENÉRICO 490</t>
-  </si>
-  <si>
-    <t>LAMPADA COMPACTA 25W 127V 3U LUZ BRANCO OUROLUX 0.024 BRANCO OUROLUX 491</t>
-  </si>
-  <si>
-    <t>CENTRI TAF PVC 03/04 DISJUNTOR BRANCO EMBALAGEM 0.048 03 BRANCO GENÉRICO 492</t>
-  </si>
-  <si>
-    <t>CENTRI TAF PVC 06/08 DISJUNTOR BRANCO EMBALAGEM 0.048 08 BRANCO GENÉRICO 480</t>
-  </si>
-  <si>
-    <t>TAF CENTRO DISTRIBUIÇÃO DISJUNTOR DIN/NEMA 03/04 EMBALAGEM FM 0.024 17.0 03 TAF 479</t>
-  </si>
-  <si>
-    <t>TAF CENTRO DISTRIBUIÇÃO DISJUNTOR DIN/NEMA 06/08 EMBALAGEM FM 0.024 20.0 08 TAF 479</t>
-  </si>
-  <si>
-    <t>CENTRI TAF PVC 12/16 DISJUNTOR BRANCO/FUME EMBALAGEM 0.048 12 BRANCO GENÉRICO 480</t>
-  </si>
-  <si>
-    <t>CAIXINHA LUZ PE 4X2 PRETO 0.031 7.0 4x2 PRETO GENÉRICO 443</t>
-  </si>
-  <si>
-    <t>CAIXINHA LUZ PE 4X2 AMARELO 0.031 7.0 4x2 AMARELO GENÉRICO 437</t>
-  </si>
-  <si>
-    <t>CAIXINHA LUZ PRETA PVC 4X4 MONDIALE 0.031 4x4 GENÉRICO 493</t>
-  </si>
-  <si>
-    <t>SUPORTE LAJE PE FIXO 30CM PRETO 0.032 6.0 PRETO GENÉRICO 494</t>
-  </si>
-  <si>
-    <t>SUPORTE LAJE PE FIXO 30CM AMARELO 0.014 11.5 AMARELO GENÉRICO 494</t>
-  </si>
-  <si>
-    <t>JNG DISJUNTOR DIN UNIPOLAR 16A CURVA C 0.024 16.0A 1P 1.8 JNG 436</t>
-  </si>
-  <si>
-    <t>JNG DISJUNTOR DIN UNIPOLAR 20A CURVA C 0.024 20.0A 1P 1.8 JNG 436</t>
-  </si>
-  <si>
-    <t>JNG DISJUNTOR DIN UNIPOLAR 25A CURVA C 0.024 25.0A 1P 1.8 JNG 436</t>
-  </si>
-  <si>
-    <t>JNG DISJUNTOR DIN UNIPOLAR 32A CURVA C 0.024 32.0A 1P 1.8 JNG 436</t>
-  </si>
-  <si>
-    <t>JNG DISJUNTOR DIN UNIPOLAR 40A CURVA C 0.024 40.0A 1P 1.8 JNG 436</t>
-  </si>
-  <si>
-    <t>JNG DISJUNTOR DIN UNIPOLAR 50A CURVA C 0.024 50.0A 1P 1.8 JNG 436</t>
-  </si>
-  <si>
-    <t>JNG DISJUNTOR DIN UNIPOLAR 63A CURVA C 0.024 63.0A 1P 2.1 JNG 436</t>
-  </si>
-  <si>
-    <t>JNG DISJUNTOR DIN BIPOLAR 06A CURVA C 0.024 2P 3.5 JNG 436</t>
-  </si>
-  <si>
-    <t>JNG DISJUNTOR DIN BIPOLAR 32A CURVA C 0.024 32.0A 2P 3.5 JNG 444</t>
-  </si>
-  <si>
-    <t>JNG DISJUNTOR DIN BIPOLAR 40A CURVA C 0.024 40.0A 2P 3.5 JNG 436</t>
-  </si>
-  <si>
-    <t>JNG DISJUNTOR DIN BIPOLAR 50A CURVA C 0.024 50.0A 2P 3.5 JNG 436</t>
-  </si>
-  <si>
-    <t>JNG DISJUNTOR DIN BIPOLAR 63A CURVA C 0.024 63.0A 2P 3.5 JNG 444</t>
-  </si>
-  <si>
-    <t>JNG BARRAMENTO DIN 2P 63A 12 POLOS 0.048 63.0A 2P 2.2 JNG 447</t>
-  </si>
-  <si>
-    <t>JNG CONECTOR GENERICO ATE 25MM CONEDZ47 0.024 25mm 2.0 JNG 495</t>
-  </si>
-  <si>
-    <t>CENTRI ILUMI PVC 1/2 DISJUNTOR BRANCO SOB 0.048 1/2" 1/2" BRANCO ILUMI 460</t>
-  </si>
-  <si>
-    <t>ILUMI PLAFONIER RED PVC SOQ PORCELANA BRANCO 0.032 14.0 BRANCO ILUMI 439</t>
-  </si>
-  <si>
-    <t>ILUMI PLAFONIER RED PVC SOQ PORCELANA PRETO 0.032 14.0 PRETO ILUMI 439</t>
-  </si>
-  <si>
-    <t>PLAFON DECORA PVC ILUMI BRANCO 0.024 BRANCO ILUMI 486</t>
-  </si>
-  <si>
-    <t>LUVA PARACOND CORRUGADO CORRER PLASTIK 3/425 0.024 PLASTIK 496</t>
-  </si>
-  <si>
-    <t>SISTEMA X ILUMI CANALETA COMDIV 20X10X2MT DF 0.024 ILUMI 497</t>
-  </si>
-  <si>
-    <t>SISTEMA X ILUMI COTOVELO LATERAL 90 BRANCO 6201 0.024 BRANCO ILUMI 498</t>
-  </si>
-  <si>
-    <t>SISTEMA X ILUMI COTOVELO INTERNO BRANCO 6202 0.024 BRANCO ILUMI 498</t>
-  </si>
-  <si>
-    <t>SISTEMA X ILUMI COTOVELO EXTERNO BRANCO 6203 0.024 BRANCO ILUMI 498</t>
-  </si>
-  <si>
-    <t>SISTEMA X ILUMI LUVA BRANCO 6205 0.024 BRANCO ILUMI 498</t>
-  </si>
-  <si>
-    <t>FOXLUX REFLETOR LED 20W ALUMINIO 6500K 0.024 12.0 FOXLUX 441</t>
-  </si>
-  <si>
-    <t>FOXLUX REFLETOR LED 50W ALUMINIO 6500K 0.024 17.0 FOXLUX 441</t>
-  </si>
-  <si>
-    <t>FOXLUX REFLETOR LED 100W ALUMINIO 6500K 0.024 19.0 FOXLUX 441</t>
-  </si>
-  <si>
-    <t>FOXLUX REFLETOR LED 150W ALUMINIO 6500K 0.024 24.0 FOXLUX 441</t>
-  </si>
-  <si>
-    <t>FOXLUX LAMPADA LED ALTA POT 20W1600LM 6500K 0.024 7.0 FOXLUX 499</t>
-  </si>
-  <si>
-    <t>FOXLUX LAMPADA LED ALTA POT 30W2400LM 6500K 0.024 5.0 FOXLUX 499</t>
-  </si>
-  <si>
-    <t>FOXLUX LAMPADA LED ALTA POT 40W3200LM 6500K 0.024 12.5 FOXLUX 499</t>
-  </si>
-  <si>
-    <t>FOXLUX LAMPADA LED A60 12W1050LM 6500K 0.024 6.0 FOXLUX 442</t>
-  </si>
-  <si>
-    <t>FOXLUX LAMPADA LED A60 15W1250LM 6500K 0.024 6.0 FOXLUX 442</t>
-  </si>
-  <si>
-    <t>FOXLUX LAMPADA HALOGENA BULBO CLASSICA 100X127 0.024 5.0 FOXLUX 500</t>
-  </si>
-  <si>
-    <t>FOXLUX FIO LUSTRE CRISTAL 2X0,75 18 R/100M 0.024 24.0 TRANSPARENTE FOXLUX 501</t>
-  </si>
-  <si>
-    <t>FOXLUX FIO SOM BICOR 2X0,75 18 R/100M 0.024 22.0 FOXLUX 501</t>
-  </si>
-  <si>
-    <t>FOXLUX LAMPADA LED A60 09W803LM 6500K 0.024 6.0 FOXLUX 490</t>
-  </si>
-  <si>
-    <t>FOXLUX PLAFONIER RED PVC SOQ PORCELANA BRANCO 4014 0.032 14.5 BRANCO FOXLUX 439</t>
-  </si>
-  <si>
-    <t>FOXLUX LAMPADA LED ALTA POT 50W4000LM 6500K 0.024 12.0 FOXLUX 499</t>
-  </si>
-  <si>
-    <t>FOXLUX LUMINARIA LED LINEAR 18W 60CM 6500K SLIM 0.024 8.0 FOXLUX 502</t>
-  </si>
-  <si>
-    <t>FOXLUX LUMINARIA LED LINEAR 36W 1,20M 6500K SLIM 0.008 1" 8.0 FOXLUX 502</t>
-  </si>
-  <si>
-    <t>ANNLUX CAPACITOR 20UF 250VAC 2 FIOS 1122 0.024 3.5 ANNLUX 503</t>
-  </si>
-  <si>
-    <t>ANNLUX PLAFONIER QUADRADO PVC SOQ BRANCO 0.056 16.5 BRANCO ANNLUX 504</t>
-  </si>
-  <si>
-    <t>ANNLUX PLAFONIER OITAVADO PVC SOQ PORCELANA BRANCO 0.056 15.0 BRANCO ANNLUX 439</t>
-  </si>
-  <si>
-    <t>SUPORTE PARADISJUNTOR DIM 10 RELUBRAS 0.008 GENÉRICO 505</t>
-  </si>
-  <si>
-    <t>INJEREST SUPORTE LAJE PE FIXO 30CM PRETO 0.048 33.0 PRETO INJEREST 494</t>
-  </si>
-  <si>
-    <t>INJEREST SUPORTE LAJE PE FIXO 30CM AMARELO 0.015 33.0 AMARELO INJEREST 494</t>
-  </si>
-  <si>
-    <t>CONDUITE CORRUGADO AMARELO FORTLEV B 3/4 RL/50 0.048 3/4" AMARELO GENÉRICO 470</t>
-  </si>
-  <si>
-    <t>CONDUITE CORRUGADO AMARELO FORTLEV C 1 RL/25 0.048 1" AMARELO GENÉRICO 470</t>
-  </si>
-  <si>
-    <t>PLAFONIER PVC DECOR OCTOGONO SOQ PORCELANA BRANCO 0.032 17.0 BRANCO GENÉRICO 439</t>
-  </si>
-  <si>
-    <t>PLAFONIER RED PVC SOQ PORCELANA BRANCO 0.032 17.0 BRANCO GENÉRICO 439</t>
-  </si>
-  <si>
-    <t>ILUMI LUMINARIA TARTARUGA FERRO/VIDRO BRANCO JR 0.008 BRANCO ILUMI 506</t>
-  </si>
-  <si>
-    <t>ILUMI LUMINARIA TARTARUGA FERRO/VIDRO PRETO JR 0.008 PRETO ILUMI 506</t>
-  </si>
-  <si>
-    <t>CONDUITE CORRUGADO AMARELO ADTEX A 1/2 RL50 0.048 1/2" AMARELO GENÉRICO 470</t>
-  </si>
-  <si>
-    <t>CONDUITE CORRUGADO AMARELO ADTEX B 3/4 RL50 0.048 3/4" AMARELO GENÉRICO 470</t>
-  </si>
-  <si>
-    <t>CONDUITE CORRUGADO AMARELO ADTEX C 1 RL25 0.048 1" AMARELO GENÉRICO 470</t>
-  </si>
-  <si>
-    <t>FOXLUX PASSA FIO 10M ALMA ACO 0.024 18.0 FOXLUX 465</t>
-  </si>
-  <si>
-    <t>FOXLUX PASSA FIO 15M ALMA ACO 0.024 18.0 FOXLUX 465</t>
-  </si>
-  <si>
-    <t>FOXLUX PASSA FIO 20M ALMA ACO 0.024 18.0 FOXLUX 465</t>
-  </si>
-  <si>
-    <t>FOXLUX PASSA FIO 30M ALMA ACO 0.024 22.0 FOXLUX 465</t>
-  </si>
-  <si>
-    <t>LUKMA DISJUNTOR DIN BIPOLAR 10A CURVA C 0.024 10.0A 2P 25.0 LUKMA 436</t>
-  </si>
-  <si>
-    <t>LUKMA DISJUNTOR DIN BIPOLAR 32A CURVA C 0.024 32.0A 2P 25.0 LUKMA 444</t>
-  </si>
-  <si>
-    <t>LUKMA DISJUNTOR DIN BIPOLAR 40A CURVA C 0.024 40.0A 2P 3.5 LUKMA 444</t>
-  </si>
-  <si>
-    <t>LUKMA DISJUNTOR DIN BIPOLAR 63A CURVA C 0.024 63.0A 2P 4.0 LUKMA 444</t>
-  </si>
-  <si>
-    <t>ARM PRESS BOW PESADA PB1 DUMON 0.024 GENÉRICO 507</t>
-  </si>
-  <si>
-    <t>CONECTOR WAGO 2P 0,14A4,0M 32A COM6 0.024 32.0A 2P WAGO 508</t>
-  </si>
-  <si>
-    <t>CONECTOR WAGO 3P 0,14A4,0M 32A COM4 0.024 32.0A 3P WAGO 449</t>
-  </si>
-  <si>
-    <t>CONECTOR WAGO 2P 05 A 6,0M 41A COM3 0.024 2P WAGO 508</t>
-  </si>
-  <si>
-    <t>ELETRODUTO ZINCADO ZETONE B 3/4X3MT 0.024 GENÉRICO 509</t>
-  </si>
-  <si>
-    <t>LUVA PARAELETRODUTO PVC PLASTBIG B 3/4 0.008 3/4" PLASTBIG 510</t>
-  </si>
-  <si>
-    <t>LUVA PARAELETRODUTO PVC PLASTBIG D 1,1/4 0.008 1" PLASTBIG 510</t>
-  </si>
-  <si>
-    <t>LUVA PARAELETRODUTO PVC PLASTBIG E 1,1/2 0.008 1" PLASTBIG 510</t>
-  </si>
-  <si>
-    <t>LUVA PARAELETRODUTO PVC PLASTBIG F 2 0.008 PLASTBIG 510</t>
-  </si>
-  <si>
-    <t>ANNLUX CAPACITOR 10UF 250VAC 2 FIOS 944 0.024 2.5 ANNLUX 503</t>
-  </si>
-  <si>
-    <t>ANNLUX CAPACITOR 16UF 250VAC 2 FIOS 923 0.024 2.5 ANNLUX 503</t>
-  </si>
-  <si>
-    <t>ANNLUX FUSIVEL DE VIDRO TIPO 3AG 5,00A 0.048 0.5 ANNLUX 511</t>
-  </si>
-  <si>
-    <t>ANNLUX FUSIVEL DE VIDRO TIPO 3AG 10,0A 0.048 0.5 ANNLUX 511</t>
-  </si>
-  <si>
-    <t>ANNLUX FUSIVEL DE VIDRO TIPO 20AG 8,00A 0.048 0.5 ANNLUX 511</t>
-  </si>
-  <si>
-    <t>ANNLUX FUSIVEL CERAMICO MICROONDAS 3AG 15,0A 0.048 0.5 ANNLUX 512</t>
-  </si>
-  <si>
-    <t>ANNLUX FUSIVEL CERAMICO MICROONDAS 3AG 20,0A 0.048 0.5 ANNLUX 512</t>
-  </si>
-  <si>
-    <t>ANNLUX FUSIVEL DE VIDRO TIPO 3AG 7,00A 0.048 0.5 ANNLUX 511</t>
-  </si>
-  <si>
-    <t>SEA CONECTOR P/ HASTE 1/23/4X5/8 0.024 1" 2.0 SEA 513</t>
-  </si>
-  <si>
-    <t>CONDUSCABOS CABO FLEXIVEL 1,50 PRETO R/100M 0.008 1" 23.0 PRETO CONDUSCABOS 466</t>
-  </si>
-  <si>
-    <t>CONDUSCABOS CABO FLEXIVEL 1,50 VERMELHO R/100M 0.008 1" 23.0 VERMELHO CONDUSCABOS 466</t>
-  </si>
-  <si>
-    <t>ELETRODUTO PVC DANTAS B 3/4 X 3MT 0.024 3/4" GENÉRICO 514</t>
-  </si>
-  <si>
-    <t>CONECTOR FERTAK PORCELANA 16MM BIF 8203 0.039 16mm FERTAK 515</t>
-  </si>
-  <si>
-    <t>CONECTOR FERTAK PORCELANA 10MM TRIF 8204 0.039 10mm FERTAK 457</t>
-  </si>
-  <si>
-    <t>LUMINARIA ALETADA COMPL 2X20 BRANCO BIVOLT LUMIART/BLUM 0.024 BRANCO GENÉRICO 516</t>
-  </si>
-  <si>
-    <t>LAMPADA LED BULBO 09W BIVOLT BLUMENAU 0.024 BLUMENAU 517</t>
-  </si>
-  <si>
-    <t>LAMPADA LED GLOBO 20W E27 6500K BV BLUMENAU 0.024 BLUMENAU 518</t>
-  </si>
-  <si>
-    <t>LAMPADA LED GLOBO 30W E27 6500K BV BLUMENAU 0.024 BLUMENAU 518</t>
-  </si>
-  <si>
-    <t>PASSA FIO MEGATRON COMALMA DE ACO 10MT 0.024 GENÉRICO 519</t>
-  </si>
-  <si>
-    <t>PASSA FIO MEGATRON COMALMA DE ACO 15MT 0.024 GENÉRICO 519</t>
-  </si>
-  <si>
-    <t>PASSA FIO MEGATRON COMALMA DE ACO 20MT 0.024 GENÉRICO 519</t>
-  </si>
-  <si>
-    <t>FIO TELEFONE CCI 01 PAR R/200M 0.008 GENÉRICO 520</t>
-  </si>
-  <si>
-    <t>MEGATRON CABO PP 0500V 2X1,5 R/100M 0.024 36.0 MEGATRON 521</t>
-  </si>
-  <si>
-    <t>NEW FIX PARAFUSO CAIXINHA LUZ PHILIPS 9/64 11/2 0.031 9.5 NEW FIX 522</t>
-  </si>
-  <si>
-    <t>NEW FIX PARAFUSO CAIXINHA LUZ PHILIPS 9/64 2 0.031 9.5 NEW FIX 522</t>
-  </si>
-  <si>
-    <t>NEW FIX PARAFUSO CAIXINHA LUZ PHILIPS 9/64 3 0.031 9.5 NEW FIX 522</t>
-  </si>
-  <si>
-    <t>AVANT LAMPADA LED ALTA POT 30W2400LM 6500K 0.024 3.0 AVANT 499</t>
-  </si>
-  <si>
-    <t>AVANT LAMPADA LED A60 15W1350LM 6500K 0.024 6.0 AVANT 490</t>
-  </si>
-  <si>
-    <t>AVANT LAMPADA LED A60 12W1050LM 6500K 0.024 6.0 AVANT 490</t>
-  </si>
-  <si>
-    <t>AVANT LAMPADA LED ALTA POT 50W4000LM 6500K 0.024 10.0 AVANT 499</t>
-  </si>
-  <si>
-    <t>AVANT LAMPADA LED ALTA POT 20W1600LM 6500K 0.024 6.0 AVANT 499</t>
-  </si>
-  <si>
-    <t>AVANT LUMINARIA EMERG 30 LEDS 100LM 11CM 0.024 5.0 AVANT 523</t>
-  </si>
-  <si>
-    <t>LUKMA BARRAMENTO DIN 2P 80A 12 POLOS 0.048 2P 25.0 LUKMA 447</t>
-  </si>
-  <si>
-    <t>LAMPADA LED BULBO 09W 6500K BIVOLT KIAN 0.024 KIAN 517</t>
-  </si>
-  <si>
-    <t>LAMPADA LED BULBO 12W 6500K BIVOLT KIAN 0.024 KIAN 524</t>
-  </si>
-  <si>
-    <t>LAMPADA LED BULBO 15W 6500K BIVOLT KIAN 0.024 KIAN 524</t>
-  </si>
-  <si>
-    <t>LAMPADA LED GLOBO 20W 6500K E27 KIAN 0.024 KIAN 518</t>
-  </si>
-  <si>
-    <t>LAMPADA LED BULBO 09W 6500K BIVOLT OUROLUX 0.024 OUROLUX 517</t>
-  </si>
-  <si>
-    <t>TERMINAL GAS 1/2 BSP F 3/8 ROCO 2017 0.024 1/2" ROCO 525</t>
-  </si>
-  <si>
-    <t>TERMINAL GAS 1/2 NPT M 3/8 ROCO 2029 0.024 1/2" ROCO 525</t>
-  </si>
-  <si>
-    <t>AVANT LAMPADA LED BOLINHA 4W AZUL 0.024 4.5 AZUL AVANT 526</t>
-  </si>
-  <si>
-    <t>AVANT LAMPADA LED BOLINHA 4W VD 0.024 5.0 AVANT 526</t>
-  </si>
-  <si>
-    <t>AVANT LAMPADA LED BOLINHA 4W VERMELHO 0.024 5.0 VERMELHO AVANT 526</t>
-  </si>
-  <si>
-    <t>AVANT LAMPADA HALOGENA BULBO CLASSICA 70X127 0.024 6.0 AVANT 500</t>
-  </si>
-  <si>
-    <t>PERFIL LIDER ELETRODUTO ZINCADO 3/4 LEVE 0.024 3/4" 1.9 PERFIL LIDER 527</t>
-  </si>
-  <si>
-    <t>LAMPADA TUBOLED 18W T08 6500K LED BEE 0.024 LED BEE 528</t>
-  </si>
-  <si>
-    <t>LAMPADA LED BULBO 09W 6500K BIVOLT LED BEE 0.024 LED BEE 517</t>
-  </si>
-  <si>
-    <t>LAMPADA LED BULBO 15W 6500K BIVOLT LED BEE 0.024 LED BEE 524</t>
-  </si>
-  <si>
-    <t>REFLETOR COMLED LED BEE 30W 6500K IP65 SMD 0.024 LED BEE 529</t>
-  </si>
-  <si>
-    <t>REFLETOR COMLED LED BEE 50W 6500K IP65 SMD 0.024 LED BEE 529</t>
-  </si>
-  <si>
-    <t>GALAXY LAMPADA LED ALTA POT 30W2400LM 6500K 0.024 7.5 GALAXY 499</t>
-  </si>
-  <si>
-    <t>GALAXY LAMPADA LED ALTA POT 40W3200LM 6500K 0.024 8.0 GALAXY 499</t>
-  </si>
-  <si>
-    <t>GALAXY LAMPADA LED ALTA POT 50W4000LM 6500K 0.024 10.0 GALAXY 499</t>
-  </si>
-  <si>
-    <t>GALAXY LAMPADA LED A60 09W803LM 6500K 0.024 6.0 GALAXY 490</t>
-  </si>
-  <si>
-    <t>GALAXY LAMPADA LED A60 12W1018LM 6500K 0.024 6.0 GALAXY 490</t>
-  </si>
-  <si>
-    <t>GALAXY LAMPADA LED ALTA POT 20W1600LM 6500K 0.024 13.5 GALAXY 499</t>
-  </si>
-  <si>
-    <t>GALAXY LAMPADA LED A60 15W1311LM 6500K 0.024 6.0 GALAXY 490</t>
-  </si>
-  <si>
-    <t>GALAXY LAMPADA LED A60 09W540LM 1000K ANTI INSETO 0.024 6.0 GALAXY 530</t>
-  </si>
-  <si>
-    <t>AIÉDEM SUPORTE DISJUNTOR DIN ALUMINIO TRILHO 20CM 35X7,5 0.048 3.5 AIÉDEM 531</t>
-  </si>
-  <si>
-    <t>JOGO SOQUETE TITANIUM 1/4 41PCS 5520 0.024 1/4" TITANIUM 532</t>
-  </si>
-  <si>
-    <t>JOGO SOQUETE TITANIUM COMCATRACA 48PC 0.024 TITANIUM 533</t>
-  </si>
-  <si>
-    <t>CONDUSCABOS CABO FLEXIVEL 1,50 AZUL R/100M 0.008 1" 23.0 AZUL CONDUSCABOS 466</t>
-  </si>
-  <si>
-    <t>ANNLUX FUSIVEL CERAMICO MICROONDAS 20AG 8,0A 0.048 0.5 ANNLUX 512</t>
-  </si>
-  <si>
-    <t>LS CHAIRA HASTE COMCABO 10 0.024 7.5 LS 534</t>
-  </si>
-  <si>
-    <t>JOGO SOQUETE FERTAK COMCATRACA 40PC 0.024 FERTAK 533</t>
-  </si>
-  <si>
-    <t>CONECTOR FERTAK PORCELANA 16MM TRIF 8205 0.039 16mm FERTAK 515</t>
-  </si>
-  <si>
-    <t>LUVA PARAELETRODUTO PVC PLASTBIG C 1 0.008 1" PLASTBIG 510</t>
-  </si>
-  <si>
-    <t>SISTEMA X RADIAL CANALETA BRANCO COMFITA 20X2MT 0.024 BRANCO RADIAL 464</t>
-  </si>
-  <si>
-    <t>CENTRI ILUMI PVC 16/24 DISJUNTOR BRANCO EMBALAGEM 0.048 BRANCO ILUMI 480</t>
-  </si>
-  <si>
-    <t>HASTE TERRA LBM 1/2X1,50MT 11,5MM 0.024 11.5mm GENÉRICO 535</t>
-  </si>
-  <si>
-    <t>LUMINARIA ALETADA PARAFL 2X20 PRETO COMREATOR BLUMENA 0.024 PRETO GENÉRICO 536</t>
-  </si>
-  <si>
-    <t>LUMINARIA ALETADA COMPL 2X20 PRETO BIVOLT LUMIART/BLUM 0.024 PRETO GENÉRICO 516</t>
-  </si>
-  <si>
-    <t>DISJUNTOR STECK SERIE SD61 50A 1P CURVA C 3KA 0.024 50.0A 1P GENÉRICO 462</t>
-  </si>
-  <si>
-    <t>DISJUNTOR STECK SERIE SD61 25A 1P CURVA C 3KA 0.024 25.0A 1P GENÉRICO 462</t>
-  </si>
-  <si>
-    <t>DISJUNTOR STECK SERIE SD61 63A 1P CURVA C 3KA 0.024 63.0A 1P GENÉRICO 462</t>
-  </si>
-  <si>
-    <t>ELETRODUTO ROSCA PVC A 1/2 0.024 1/2" GENÉRICO 537</t>
-  </si>
-  <si>
-    <t>ELETRODUTO ROSCA PVC B 3/4 0.024 3/4" GENÉRICO 514</t>
-  </si>
-  <si>
-    <t>RECEPTACULO CANIELLO LATAO F 519 0.024 GENÉRICO 476</t>
-  </si>
-  <si>
-    <t>LAMPADA HALOGENA BULBO CLASSICA 120X220 0.024 GENÉRICO 500</t>
+    <t>TRAMONTINA CAIXA LUZ AMARELO</t>
+  </si>
+  <si>
+    <t>FC CAIXINHA LUZ PVC AMARELO</t>
+  </si>
+  <si>
+    <t>KRONA LUVA CORRUGADO C 3/4</t>
+  </si>
+  <si>
+    <t>INJEREST CAIXINHA LUZ PE PRETO</t>
+  </si>
+  <si>
+    <t>SCHNEIDER BARRAMENTO DIN 80A 12 POLOS EZ9X33112</t>
+  </si>
+  <si>
+    <t>SCHNEIDER BARRAMENTO DIN 80A 12 POLOS EZ9X33212</t>
+  </si>
+  <si>
+    <t>CONECTOR WAGO 08 A 4,0M 32A</t>
+  </si>
+  <si>
+    <t>CONECTOR PORCELANA COM100 BRASFORT</t>
+  </si>
+  <si>
+    <t>CONECTOR PORCELANA COM12 BRASFORT</t>
+  </si>
+  <si>
+    <t>THOMPSON CONECTOR 03 BORNE</t>
+  </si>
+  <si>
+    <t>TRAMONTINA CAIXINHA LUZ PVC AMARELO /044</t>
+  </si>
+  <si>
+    <t>TRAMONTINA CORRUGADO PVC AMARELO METRO/50</t>
+  </si>
+  <si>
+    <t>TRAMONTINA CAIXINHA LUZ DRYWALL AMARELO /071</t>
+  </si>
+  <si>
+    <t>CAIXINHA LUZ AMARELA TRAMONTINA</t>
+  </si>
+  <si>
+    <t>TRAMONTINA CAIXINHA LUZ PVC AMARELO /043</t>
+  </si>
+  <si>
+    <t>TRAMONTINA CORRUGADO PVC AMARELO METRO/25</t>
+  </si>
+  <si>
+    <t>CONECTOR INTERNEED PORCELANA TRIF</t>
+  </si>
+  <si>
+    <t>STECK BARRAMENTO DIN 80A 12 POLOS 2F210B</t>
+  </si>
+  <si>
+    <t>CENTRI STECK PVC DISJUNTOR DIN SOB BRANCO SCT4</t>
+  </si>
+  <si>
+    <t>CENTRI STECK PVC DISJUNTOR DIN SOB BRANCO SCT2</t>
+  </si>
+  <si>
+    <t>CENTRI STECK PVC DISJUNTOR DIN EMBALAGEM BRANCO</t>
+  </si>
+  <si>
+    <t>STECK CENTRO DISTRIBUIÇÃO DISJUNTOR DIN EMBALAGEM BRANCO</t>
+  </si>
+  <si>
+    <t>DISJUNTOR STECK SERIE SD61 16A CURVA C 3KA</t>
+  </si>
+  <si>
+    <t>DISJUNTOR STECK SERIE SD61 20A CURVA C 3KA</t>
+  </si>
+  <si>
+    <t>DISJUNTOR STECK SERIE SD61 40A CURVA C 3KA</t>
+  </si>
+  <si>
+    <t>DISJUNTOR STECK SERIE SD62 40A CURVA C 3KA</t>
+  </si>
+  <si>
+    <t>DISJUNTOR STECK SERIE SD62 50A CURVA C 3KA</t>
+  </si>
+  <si>
+    <t>BIKI CENTRO DISTRIBUIÇÃO DISJUNTOR DIN/NEMA /04 EMBALAGEM BRANCO</t>
+  </si>
+  <si>
+    <t>PENZEL TERM PREISOL PINO AMARELO /6,00MM C13MM</t>
+  </si>
+  <si>
+    <t>THOMPSON CENTRO DISTRIBUIÇÃO DISJUNTOR DIN/NEMA 06/ EMBALAGEM CINZA</t>
+  </si>
+  <si>
+    <t>THOMPSOM CENTRI PVC /16 DISJUNTOR BRANCO/FUME EMBALAGEM</t>
+  </si>
+  <si>
+    <t>THOMPSOM CENTRI PVC 06/ DISJUNTOR BRANCO EMBALAGEM</t>
+  </si>
+  <si>
+    <t>THOMPSOM CENTRI PVC /16 DISJUNTOR BRANCO EMBALAGEM</t>
+  </si>
+  <si>
+    <t>CENTRI ILUMI PVC /16 DISJUNTOR BRANCO EMBALAGEM</t>
+  </si>
+  <si>
+    <t>CENTRI TAF PVC /04 DISJUNTOR BRANCO EMBALAGEM</t>
+  </si>
+  <si>
+    <t>CENTRI TAF PVC 06/ DISJUNTOR BRANCO EMBALAGEM</t>
+  </si>
+  <si>
+    <t>TAF CENTRO DISTRIBUIÇÃO DISJUNTOR DIN/NEMA /04 EMBALAGEM FM</t>
+  </si>
+  <si>
+    <t>TAF CENTRO DISTRIBUIÇÃO DISJUNTOR DIN/NEMA 06/ EMBALAGEM FM</t>
+  </si>
+  <si>
+    <t>CENTRI TAF PVC /16 DISJUNTOR BRANCO/FUME EMBALAGEM</t>
+  </si>
+  <si>
+    <t>CAIXINHA LUZ PE PRETO</t>
+  </si>
+  <si>
+    <t>CAIXINHA LUZ PE AMARELO</t>
+  </si>
+  <si>
+    <t>CAIXINHA LUZ PRETA PVC MONDIALE</t>
+  </si>
+  <si>
+    <t>JNG BARRAMENTO DIN 63A 12 POLOS</t>
+  </si>
+  <si>
+    <t>JNG CONECTOR GENERICO ATE CONEDZ47</t>
+  </si>
+  <si>
+    <t>CONECTOR WAGO 0,14A4,0M 32A COM6</t>
+  </si>
+  <si>
+    <t>CONECTOR WAGO 0,14A4,0M 32A COM4</t>
+  </si>
+  <si>
+    <t>CONECTOR WAGO 05 A 6,0M 41A COM3</t>
+  </si>
+  <si>
+    <t>CONECTOR FERTAK PORCELANA BIF 8203</t>
+  </si>
+  <si>
+    <t>CONECTOR FERTAK PORCELANA TRIF 8204</t>
+  </si>
+  <si>
+    <t>LUKMA BARRAMENTO DIN 80A 12 POLOS</t>
+  </si>
+  <si>
+    <t>CONECTOR FERTAK PORCELANA TRIF 8205</t>
+  </si>
+  <si>
+    <t>DISJUNTOR STECK SERIE SD61 50A CURVA C 3KA</t>
+  </si>
+  <si>
+    <t>DISJUNTOR STECK SERIE SD61 25A CURVA C 3KA</t>
+  </si>
+  <si>
+    <t>DISJUNTOR STECK SERIE SD61 63A CURVA C 3KA</t>
+  </si>
+  <si>
+    <t>3/4" 1.0</t>
+  </si>
+  <si>
+    <t>1/2" 1.0</t>
+  </si>
+  <si>
+    <t>1.0 4x2</t>
+  </si>
+  <si>
+    <t>1.0</t>
+  </si>
+  <si>
+    <t>1P 10.0A 8.0</t>
+  </si>
+  <si>
+    <t>2P 40.0A 8.0</t>
+  </si>
+  <si>
+    <t>2P 50.0A 8.0</t>
+  </si>
+  <si>
+    <t>11.0 4x4</t>
+  </si>
+  <si>
+    <t>25mm 3.0</t>
+  </si>
+  <si>
+    <t>14.0</t>
+  </si>
+  <si>
+    <t>4.5</t>
+  </si>
+  <si>
+    <t>19.0</t>
+  </si>
+  <si>
+    <t>3.0</t>
+  </si>
+  <si>
+    <t>5.0 4x2</t>
+  </si>
+  <si>
+    <t>2P 50.0A 25.0</t>
+  </si>
+  <si>
+    <t>5.0</t>
+  </si>
+  <si>
+    <t>3.5</t>
+  </si>
+  <si>
+    <t>1P 3.0</t>
+  </si>
+  <si>
+    <t>2P 3.0</t>
+  </si>
+  <si>
+    <t>3P 32.0A</t>
+  </si>
+  <si>
+    <t>2P 32.0A</t>
+  </si>
+  <si>
+    <t>1" 1.0</t>
+  </si>
+  <si>
+    <t>3P 6mm 1.0</t>
+  </si>
+  <si>
+    <t>3P 16mm 1.0</t>
+  </si>
+  <si>
+    <t>1P 20.0A 8.0</t>
+  </si>
+  <si>
+    <t>200.0</t>
+  </si>
+  <si>
+    <t>10mm 20.0</t>
+  </si>
+  <si>
+    <t>16mm 2.5</t>
+  </si>
+  <si>
+    <t>0.39</t>
+  </si>
+  <si>
+    <t>25mm 50.0</t>
+  </si>
+  <si>
+    <t>9.0 3x3</t>
+  </si>
+  <si>
+    <t>32mm 3.0</t>
+  </si>
+  <si>
+    <t>14.5</t>
+  </si>
+  <si>
+    <t>1P 23.0 08</t>
+  </si>
+  <si>
+    <t>1P 16.0A</t>
+  </si>
+  <si>
+    <t>1P 20.0A</t>
+  </si>
+  <si>
+    <t>1P 25.0A 8.0</t>
+  </si>
+  <si>
+    <t>1P 32.0A 8.0</t>
+  </si>
+  <si>
+    <t>1P 40.0A</t>
+  </si>
+  <si>
+    <t>2P 10.0A 8.0</t>
+  </si>
+  <si>
+    <t>2P 32.0A 8.0</t>
+  </si>
+  <si>
+    <t>2P 40.0A</t>
+  </si>
+  <si>
+    <t>2P 50.0A</t>
+  </si>
+  <si>
+    <t>2P 63.0A 8.0</t>
+  </si>
+  <si>
+    <t>14.0 03</t>
+  </si>
+  <si>
+    <t>15.0</t>
+  </si>
+  <si>
+    <t>7.0 4x2</t>
+  </si>
+  <si>
+    <t>16.5</t>
+  </si>
+  <si>
+    <t>1" 22.0</t>
+  </si>
+  <si>
+    <t>1" 23.0</t>
+  </si>
+  <si>
+    <t>1.5mm 1.5</t>
+  </si>
+  <si>
+    <t>4mm 1.0</t>
+  </si>
+  <si>
+    <t>0.5mm 11.5</t>
+  </si>
+  <si>
+    <t>1.5mm 11.5</t>
+  </si>
+  <si>
+    <t>24.0</t>
+  </si>
+  <si>
+    <t>25.0 08</t>
+  </si>
+  <si>
+    <t>4.0</t>
+  </si>
+  <si>
+    <t>13.0</t>
+  </si>
+  <si>
+    <t>11.0</t>
+  </si>
+  <si>
+    <t>17.0 03</t>
+  </si>
+  <si>
+    <t>20.0 08</t>
+  </si>
+  <si>
+    <t>6.0</t>
+  </si>
+  <si>
+    <t>11.5</t>
+  </si>
+  <si>
+    <t>1P 16.0A 1.8</t>
+  </si>
+  <si>
+    <t>1P 20.0A 1.8</t>
+  </si>
+  <si>
+    <t>1P 25.0A 1.8</t>
+  </si>
+  <si>
+    <t>1P 32.0A 1.8</t>
+  </si>
+  <si>
+    <t>1P 40.0A 1.8</t>
+  </si>
+  <si>
+    <t>1P 50.0A 1.8</t>
+  </si>
+  <si>
+    <t>1P 63.0A 2.1</t>
+  </si>
+  <si>
+    <t>2P 3.5</t>
+  </si>
+  <si>
+    <t>2P 32.0A 3.5</t>
+  </si>
+  <si>
+    <t>2P 40.0A 3.5</t>
+  </si>
+  <si>
+    <t>2P 50.0A 3.5</t>
+  </si>
+  <si>
+    <t>2P 63.0A 3.5</t>
+  </si>
+  <si>
+    <t>2P 63.0A 2.2</t>
+  </si>
+  <si>
+    <t>25mm 2.0</t>
+  </si>
+  <si>
+    <t>1/2" 1/2"</t>
+  </si>
+  <si>
+    <t>12.0</t>
+  </si>
+  <si>
+    <t>17.0</t>
+  </si>
+  <si>
+    <t>7.0</t>
+  </si>
+  <si>
+    <t>12.5</t>
+  </si>
+  <si>
+    <t>22.0</t>
+  </si>
+  <si>
+    <t>8.0</t>
+  </si>
+  <si>
+    <t>1" 8.0</t>
+  </si>
+  <si>
+    <t>33.0</t>
+  </si>
+  <si>
+    <t>18.0</t>
+  </si>
+  <si>
+    <t>2P 10.0A 25.0</t>
+  </si>
+  <si>
+    <t>2P 32.0A 25.0</t>
+  </si>
+  <si>
+    <t>2P 63.0A 4.0</t>
+  </si>
+  <si>
+    <t>2.5</t>
+  </si>
+  <si>
+    <t>0.5</t>
+  </si>
+  <si>
+    <t>1" 2.0</t>
+  </si>
+  <si>
+    <t>36.0</t>
+  </si>
+  <si>
+    <t>9.5</t>
+  </si>
+  <si>
+    <t>10.0</t>
+  </si>
+  <si>
+    <t>2P 25.0</t>
+  </si>
+  <si>
+    <t>3/4" 1.9</t>
+  </si>
+  <si>
+    <t>7.5</t>
+  </si>
+  <si>
+    <t>13.5</t>
+  </si>
+  <si>
+    <t>1P 50.0A</t>
+  </si>
+  <si>
+    <t>1P 25.0A</t>
+  </si>
+  <si>
+    <t>1P 63.0A</t>
   </si>
 </sst>
 </file>
@@ -2441,8 +2057,11 @@
       <c r="K2">
         <v>432</v>
       </c>
+      <c r="L2" t="s">
+        <v>13</v>
+      </c>
       <c r="M2" t="s">
-        <v>383</v>
+        <v>437</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -2467,8 +2086,11 @@
       <c r="K3">
         <v>433</v>
       </c>
+      <c r="L3" t="s">
+        <v>14</v>
+      </c>
       <c r="M3" t="s">
-        <v>384</v>
+        <v>438</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -2493,8 +2115,11 @@
       <c r="K4">
         <v>434</v>
       </c>
+      <c r="L4" t="s">
+        <v>383</v>
+      </c>
       <c r="M4" t="s">
-        <v>385</v>
+        <v>439</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -2516,8 +2141,11 @@
       <c r="K5">
         <v>435</v>
       </c>
+      <c r="L5" t="s">
+        <v>16</v>
+      </c>
       <c r="M5" t="s">
-        <v>386</v>
+        <v>440</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -2542,8 +2170,11 @@
       <c r="K6">
         <v>436</v>
       </c>
+      <c r="L6" t="s">
+        <v>17</v>
+      </c>
       <c r="M6" t="s">
-        <v>387</v>
+        <v>441</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -2568,8 +2199,11 @@
       <c r="K7">
         <v>436</v>
       </c>
+      <c r="L7" t="s">
+        <v>18</v>
+      </c>
       <c r="M7" t="s">
-        <v>388</v>
+        <v>442</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -2594,8 +2228,11 @@
       <c r="K8">
         <v>436</v>
       </c>
+      <c r="L8" t="s">
+        <v>19</v>
+      </c>
       <c r="M8" t="s">
-        <v>389</v>
+        <v>443</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -2620,8 +2257,11 @@
       <c r="K9">
         <v>437</v>
       </c>
+      <c r="L9" t="s">
+        <v>384</v>
+      </c>
       <c r="M9" t="s">
-        <v>390</v>
+        <v>444</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -2643,8 +2283,11 @@
       <c r="K10">
         <v>438</v>
       </c>
+      <c r="L10" t="s">
+        <v>385</v>
+      </c>
       <c r="M10" t="s">
-        <v>391</v>
+        <v>445</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -2666,8 +2309,11 @@
       <c r="K11">
         <v>439</v>
       </c>
+      <c r="L11" t="s">
+        <v>22</v>
+      </c>
       <c r="M11" t="s">
-        <v>392</v>
+        <v>446</v>
       </c>
     </row>
     <row r="12" spans="1:13">
@@ -2686,8 +2332,11 @@
       <c r="K12">
         <v>440</v>
       </c>
+      <c r="L12" t="s">
+        <v>23</v>
+      </c>
       <c r="M12" t="s">
-        <v>393</v>
+        <v>447</v>
       </c>
     </row>
     <row r="13" spans="1:13">
@@ -2706,8 +2355,11 @@
       <c r="K13">
         <v>441</v>
       </c>
+      <c r="L13" t="s">
+        <v>24</v>
+      </c>
       <c r="M13" t="s">
-        <v>394</v>
+        <v>448</v>
       </c>
     </row>
     <row r="14" spans="1:13">
@@ -2726,8 +2378,11 @@
       <c r="K14">
         <v>442</v>
       </c>
+      <c r="L14" t="s">
+        <v>25</v>
+      </c>
       <c r="M14" t="s">
-        <v>395</v>
+        <v>449</v>
       </c>
     </row>
     <row r="15" spans="1:13">
@@ -2752,8 +2407,11 @@
       <c r="K15">
         <v>443</v>
       </c>
+      <c r="L15" t="s">
+        <v>386</v>
+      </c>
       <c r="M15" t="s">
-        <v>396</v>
+        <v>450</v>
       </c>
     </row>
     <row r="16" spans="1:13">
@@ -2778,8 +2436,11 @@
       <c r="K16">
         <v>432</v>
       </c>
+      <c r="L16" t="s">
+        <v>27</v>
+      </c>
       <c r="M16" t="s">
-        <v>397</v>
+        <v>438</v>
       </c>
     </row>
     <row r="17" spans="1:13">
@@ -2804,8 +2465,11 @@
       <c r="K17">
         <v>444</v>
       </c>
+      <c r="L17" t="s">
+        <v>28</v>
+      </c>
       <c r="M17" t="s">
-        <v>398</v>
+        <v>451</v>
       </c>
     </row>
     <row r="18" spans="1:13">
@@ -2830,8 +2494,11 @@
       <c r="K18">
         <v>433</v>
       </c>
+      <c r="L18" t="s">
+        <v>29</v>
+      </c>
       <c r="M18" t="s">
-        <v>399</v>
+        <v>437</v>
       </c>
     </row>
     <row r="19" spans="1:13">
@@ -2850,8 +2517,11 @@
       <c r="K19">
         <v>445</v>
       </c>
+      <c r="L19" t="s">
+        <v>30</v>
+      </c>
       <c r="M19" t="s">
-        <v>400</v>
+        <v>452</v>
       </c>
     </row>
     <row r="20" spans="1:13">
@@ -2870,8 +2540,11 @@
       <c r="K20">
         <v>446</v>
       </c>
+      <c r="L20" t="s">
+        <v>31</v>
+      </c>
       <c r="M20" t="s">
-        <v>401</v>
+        <v>453</v>
       </c>
     </row>
     <row r="21" spans="1:13">
@@ -2893,8 +2566,11 @@
       <c r="K21">
         <v>447</v>
       </c>
+      <c r="L21" t="s">
+        <v>387</v>
+      </c>
       <c r="M21" t="s">
-        <v>402</v>
+        <v>454</v>
       </c>
     </row>
     <row r="22" spans="1:13">
@@ -2916,8 +2592,11 @@
       <c r="K22">
         <v>447</v>
       </c>
+      <c r="L22" t="s">
+        <v>388</v>
+      </c>
       <c r="M22" t="s">
-        <v>403</v>
+        <v>455</v>
       </c>
     </row>
     <row r="23" spans="1:13">
@@ -2933,8 +2612,8 @@
       <c r="K23">
         <v>448</v>
       </c>
-      <c r="M23" t="s">
-        <v>404</v>
+      <c r="L23" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="24" spans="1:13">
@@ -2956,8 +2635,11 @@
       <c r="K24">
         <v>449</v>
       </c>
+      <c r="L24" t="s">
+        <v>389</v>
+      </c>
       <c r="M24" t="s">
-        <v>405</v>
+        <v>456</v>
       </c>
     </row>
     <row r="25" spans="1:13">
@@ -2979,8 +2661,11 @@
       <c r="K25">
         <v>449</v>
       </c>
+      <c r="L25" t="s">
+        <v>389</v>
+      </c>
       <c r="M25" t="s">
-        <v>406</v>
+        <v>457</v>
       </c>
     </row>
     <row r="26" spans="1:13">
@@ -3005,8 +2690,11 @@
       <c r="K26">
         <v>433</v>
       </c>
+      <c r="L26" t="s">
+        <v>37</v>
+      </c>
       <c r="M26" t="s">
-        <v>407</v>
+        <v>458</v>
       </c>
     </row>
     <row r="27" spans="1:13">
@@ -3031,8 +2719,11 @@
       <c r="K27">
         <v>433</v>
       </c>
+      <c r="L27" t="s">
+        <v>38</v>
+      </c>
       <c r="M27" t="s">
-        <v>408</v>
+        <v>437</v>
       </c>
     </row>
     <row r="28" spans="1:13">
@@ -3057,8 +2748,11 @@
       <c r="K28">
         <v>450</v>
       </c>
+      <c r="L28" t="s">
+        <v>390</v>
+      </c>
       <c r="M28" t="s">
-        <v>409</v>
+        <v>459</v>
       </c>
     </row>
     <row r="29" spans="1:13">
@@ -3083,8 +2777,11 @@
       <c r="K29">
         <v>450</v>
       </c>
+      <c r="L29" t="s">
+        <v>391</v>
+      </c>
       <c r="M29" t="s">
-        <v>410</v>
+        <v>460</v>
       </c>
     </row>
     <row r="30" spans="1:13">
@@ -3109,8 +2806,11 @@
       <c r="K30">
         <v>436</v>
       </c>
+      <c r="L30" t="s">
+        <v>41</v>
+      </c>
       <c r="M30" t="s">
-        <v>411</v>
+        <v>461</v>
       </c>
     </row>
     <row r="31" spans="1:13">
@@ -3132,8 +2832,11 @@
       <c r="K31">
         <v>451</v>
       </c>
+      <c r="L31" t="s">
+        <v>42</v>
+      </c>
       <c r="M31" t="s">
-        <v>412</v>
+        <v>462</v>
       </c>
     </row>
     <row r="32" spans="1:13">
@@ -3152,8 +2855,11 @@
       <c r="K32">
         <v>452</v>
       </c>
+      <c r="L32" t="s">
+        <v>43</v>
+      </c>
       <c r="M32" t="s">
-        <v>413</v>
+        <v>449</v>
       </c>
     </row>
     <row r="33" spans="1:13">
@@ -3175,8 +2881,11 @@
       <c r="K33">
         <v>453</v>
       </c>
+      <c r="L33" t="s">
+        <v>392</v>
+      </c>
       <c r="M33" t="s">
-        <v>414</v>
+        <v>463</v>
       </c>
     </row>
     <row r="34" spans="1:13">
@@ -3198,8 +2907,11 @@
       <c r="K34">
         <v>453</v>
       </c>
+      <c r="L34" t="s">
+        <v>392</v>
+      </c>
       <c r="M34" t="s">
-        <v>415</v>
+        <v>464</v>
       </c>
     </row>
     <row r="35" spans="1:13">
@@ -3221,8 +2933,11 @@
       <c r="K35">
         <v>454</v>
       </c>
+      <c r="L35" t="s">
+        <v>46</v>
+      </c>
       <c r="M35" t="s">
-        <v>416</v>
+        <v>465</v>
       </c>
     </row>
     <row r="36" spans="1:13">
@@ -3238,8 +2953,8 @@
       <c r="K36">
         <v>455</v>
       </c>
-      <c r="M36" t="s">
-        <v>417</v>
+      <c r="L36" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="37" spans="1:13">
@@ -3264,8 +2979,11 @@
       <c r="K37">
         <v>434</v>
       </c>
+      <c r="L37" t="s">
+        <v>393</v>
+      </c>
       <c r="M37" t="s">
-        <v>418</v>
+        <v>450</v>
       </c>
     </row>
     <row r="38" spans="1:13">
@@ -3290,8 +3008,11 @@
       <c r="K38">
         <v>456</v>
       </c>
+      <c r="L38" t="s">
+        <v>394</v>
+      </c>
       <c r="M38" t="s">
-        <v>419</v>
+        <v>466</v>
       </c>
     </row>
     <row r="39" spans="1:13">
@@ -3316,8 +3037,11 @@
       <c r="K39">
         <v>434</v>
       </c>
+      <c r="L39" t="s">
+        <v>395</v>
+      </c>
       <c r="M39" t="s">
-        <v>420</v>
+        <v>450</v>
       </c>
     </row>
     <row r="40" spans="1:13">
@@ -3336,8 +3060,11 @@
       <c r="K40">
         <v>434</v>
       </c>
+      <c r="L40" t="s">
+        <v>396</v>
+      </c>
       <c r="M40" t="s">
-        <v>421</v>
+        <v>317</v>
       </c>
     </row>
     <row r="41" spans="1:13">
@@ -3362,8 +3089,11 @@
       <c r="K41">
         <v>434</v>
       </c>
+      <c r="L41" t="s">
+        <v>397</v>
+      </c>
       <c r="M41" t="s">
-        <v>422</v>
+        <v>467</v>
       </c>
     </row>
     <row r="42" spans="1:13">
@@ -3388,8 +3118,11 @@
       <c r="K42">
         <v>456</v>
       </c>
+      <c r="L42" t="s">
+        <v>398</v>
+      </c>
       <c r="M42" t="s">
-        <v>423</v>
+        <v>468</v>
       </c>
     </row>
     <row r="43" spans="1:13">
@@ -3411,8 +3144,11 @@
       <c r="K43">
         <v>439</v>
       </c>
+      <c r="L43" t="s">
+        <v>54</v>
+      </c>
       <c r="M43" t="s">
-        <v>424</v>
+        <v>469</v>
       </c>
     </row>
     <row r="44" spans="1:13">
@@ -3431,8 +3167,11 @@
       <c r="K44">
         <v>457</v>
       </c>
+      <c r="L44" t="s">
+        <v>399</v>
+      </c>
       <c r="M44" t="s">
-        <v>425</v>
+        <v>307</v>
       </c>
     </row>
     <row r="45" spans="1:13">
@@ -3448,8 +3187,8 @@
       <c r="K45">
         <v>458</v>
       </c>
-      <c r="M45" t="s">
-        <v>426</v>
+      <c r="L45" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="46" spans="1:13">
@@ -3471,8 +3210,11 @@
       <c r="K46">
         <v>459</v>
       </c>
+      <c r="L46" t="s">
+        <v>400</v>
+      </c>
       <c r="M46" t="s">
-        <v>427</v>
+        <v>455</v>
       </c>
     </row>
     <row r="47" spans="1:13">
@@ -3494,8 +3236,11 @@
       <c r="K47">
         <v>460</v>
       </c>
+      <c r="L47" t="s">
+        <v>401</v>
+      </c>
       <c r="M47" t="s">
-        <v>428</v>
+        <v>319</v>
       </c>
     </row>
     <row r="48" spans="1:13">
@@ -3517,8 +3262,11 @@
       <c r="K48">
         <v>460</v>
       </c>
+      <c r="L48" t="s">
+        <v>402</v>
+      </c>
       <c r="M48" t="s">
-        <v>429</v>
+        <v>320</v>
       </c>
     </row>
     <row r="49" spans="1:13">
@@ -3540,8 +3288,11 @@
       <c r="K49">
         <v>460</v>
       </c>
+      <c r="L49" t="s">
+        <v>403</v>
+      </c>
       <c r="M49" t="s">
-        <v>430</v>
+        <v>321</v>
       </c>
     </row>
     <row r="50" spans="1:13">
@@ -3569,8 +3320,11 @@
       <c r="K50">
         <v>461</v>
       </c>
+      <c r="L50" t="s">
+        <v>404</v>
+      </c>
       <c r="M50" t="s">
-        <v>431</v>
+        <v>470</v>
       </c>
     </row>
     <row r="51" spans="1:13">
@@ -3592,8 +3346,11 @@
       <c r="K51">
         <v>462</v>
       </c>
+      <c r="L51" t="s">
+        <v>405</v>
+      </c>
       <c r="M51" t="s">
-        <v>432</v>
+        <v>471</v>
       </c>
     </row>
     <row r="52" spans="1:13">
@@ -3615,8 +3372,11 @@
       <c r="K52">
         <v>462</v>
       </c>
+      <c r="L52" t="s">
+        <v>406</v>
+      </c>
       <c r="M52" t="s">
-        <v>433</v>
+        <v>472</v>
       </c>
     </row>
     <row r="53" spans="1:13">
@@ -3641,8 +3401,11 @@
       <c r="K53">
         <v>436</v>
       </c>
+      <c r="L53" t="s">
+        <v>64</v>
+      </c>
       <c r="M53" t="s">
-        <v>434</v>
+        <v>473</v>
       </c>
     </row>
     <row r="54" spans="1:13">
@@ -3667,8 +3430,11 @@
       <c r="K54">
         <v>436</v>
       </c>
+      <c r="L54" t="s">
+        <v>65</v>
+      </c>
       <c r="M54" t="s">
-        <v>435</v>
+        <v>474</v>
       </c>
     </row>
     <row r="55" spans="1:13">
@@ -3690,8 +3456,11 @@
       <c r="K55">
         <v>462</v>
       </c>
+      <c r="L55" t="s">
+        <v>407</v>
+      </c>
       <c r="M55" t="s">
-        <v>436</v>
+        <v>475</v>
       </c>
     </row>
     <row r="56" spans="1:13">
@@ -3716,8 +3485,11 @@
       <c r="K56">
         <v>436</v>
       </c>
+      <c r="L56" t="s">
+        <v>67</v>
+      </c>
       <c r="M56" t="s">
-        <v>437</v>
+        <v>476</v>
       </c>
     </row>
     <row r="57" spans="1:13">
@@ -3742,8 +3514,11 @@
       <c r="K57">
         <v>436</v>
       </c>
+      <c r="L57" t="s">
+        <v>68</v>
+      </c>
       <c r="M57" t="s">
-        <v>438</v>
+        <v>477</v>
       </c>
     </row>
     <row r="58" spans="1:13">
@@ -3765,8 +3540,11 @@
       <c r="K58">
         <v>462</v>
       </c>
+      <c r="L58" t="s">
+        <v>408</v>
+      </c>
       <c r="M58" t="s">
-        <v>439</v>
+        <v>478</v>
       </c>
     </row>
     <row r="59" spans="1:13">
@@ -3788,8 +3566,11 @@
       <c r="K59">
         <v>462</v>
       </c>
+      <c r="L59" t="s">
+        <v>409</v>
+      </c>
       <c r="M59" t="s">
-        <v>440</v>
+        <v>479</v>
       </c>
     </row>
     <row r="60" spans="1:13">
@@ -3814,8 +3595,11 @@
       <c r="K60">
         <v>436</v>
       </c>
+      <c r="L60" t="s">
+        <v>71</v>
+      </c>
       <c r="M60" t="s">
-        <v>441</v>
+        <v>480</v>
       </c>
     </row>
     <row r="61" spans="1:13">
@@ -3834,8 +3618,8 @@
       <c r="K61">
         <v>454</v>
       </c>
-      <c r="M61" t="s">
-        <v>442</v>
+      <c r="L61" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="62" spans="1:13">
@@ -3854,8 +3638,11 @@
       <c r="K62">
         <v>463</v>
       </c>
+      <c r="L62" t="s">
+        <v>73</v>
+      </c>
       <c r="M62" t="s">
-        <v>443</v>
+        <v>304</v>
       </c>
     </row>
     <row r="63" spans="1:13">
@@ -3877,8 +3664,11 @@
       <c r="K63">
         <v>454</v>
       </c>
+      <c r="L63" t="s">
+        <v>74</v>
+      </c>
       <c r="M63" t="s">
-        <v>444</v>
+        <v>462</v>
       </c>
     </row>
     <row r="64" spans="1:13">
@@ -3897,8 +3687,8 @@
       <c r="K64">
         <v>464</v>
       </c>
-      <c r="M64" t="s">
-        <v>445</v>
+      <c r="L64" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="65" spans="1:13">
@@ -3917,8 +3707,8 @@
       <c r="K65">
         <v>464</v>
       </c>
-      <c r="M65" t="s">
-        <v>446</v>
+      <c r="L65" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="66" spans="1:13">
@@ -3943,8 +3733,11 @@
       <c r="K66">
         <v>461</v>
       </c>
+      <c r="L66" t="s">
+        <v>410</v>
+      </c>
       <c r="M66" t="s">
-        <v>447</v>
+        <v>481</v>
       </c>
     </row>
     <row r="67" spans="1:13">
@@ -3966,8 +3759,11 @@
       <c r="K67">
         <v>439</v>
       </c>
+      <c r="L67" t="s">
+        <v>78</v>
+      </c>
       <c r="M67" t="s">
-        <v>448</v>
+        <v>482</v>
       </c>
     </row>
     <row r="68" spans="1:13">
@@ -3989,8 +3785,11 @@
       <c r="K68">
         <v>439</v>
       </c>
+      <c r="L68" t="s">
+        <v>79</v>
+      </c>
       <c r="M68" t="s">
-        <v>449</v>
+        <v>469</v>
       </c>
     </row>
     <row r="69" spans="1:13">
@@ -4015,8 +3814,11 @@
       <c r="K69">
         <v>437</v>
       </c>
+      <c r="L69" t="s">
+        <v>384</v>
+      </c>
       <c r="M69" t="s">
-        <v>450</v>
+        <v>483</v>
       </c>
     </row>
     <row r="70" spans="1:13">
@@ -4035,8 +3837,11 @@
       <c r="K70">
         <v>465</v>
       </c>
+      <c r="L70" t="s">
+        <v>81</v>
+      </c>
       <c r="M70" t="s">
-        <v>451</v>
+        <v>484</v>
       </c>
     </row>
     <row r="71" spans="1:13">
@@ -4061,8 +3866,11 @@
       <c r="K71">
         <v>466</v>
       </c>
+      <c r="L71" t="s">
+        <v>82</v>
+      </c>
       <c r="M71" t="s">
-        <v>452</v>
+        <v>485</v>
       </c>
     </row>
     <row r="72" spans="1:13">
@@ -4084,8 +3892,11 @@
       <c r="K72">
         <v>467</v>
       </c>
+      <c r="L72" t="s">
+        <v>83</v>
+      </c>
       <c r="M72" t="s">
-        <v>453</v>
+        <v>309</v>
       </c>
     </row>
     <row r="73" spans="1:13">
@@ -4107,8 +3918,11 @@
       <c r="K73">
         <v>467</v>
       </c>
+      <c r="L73" t="s">
+        <v>84</v>
+      </c>
       <c r="M73" t="s">
-        <v>454</v>
+        <v>309</v>
       </c>
     </row>
     <row r="74" spans="1:13">
@@ -4130,8 +3944,11 @@
       <c r="K74">
         <v>467</v>
       </c>
+      <c r="L74" t="s">
+        <v>85</v>
+      </c>
       <c r="M74" t="s">
-        <v>455</v>
+        <v>309</v>
       </c>
     </row>
     <row r="75" spans="1:13">
@@ -4153,8 +3970,11 @@
       <c r="K75">
         <v>468</v>
       </c>
+      <c r="L75" t="s">
+        <v>86</v>
+      </c>
       <c r="M75" t="s">
-        <v>456</v>
+        <v>310</v>
       </c>
     </row>
     <row r="76" spans="1:13">
@@ -4179,8 +3999,11 @@
       <c r="K76">
         <v>466</v>
       </c>
+      <c r="L76" t="s">
+        <v>87</v>
+      </c>
       <c r="M76" t="s">
-        <v>457</v>
+        <v>486</v>
       </c>
     </row>
     <row r="77" spans="1:13">
@@ -4196,8 +4019,8 @@
       <c r="K77">
         <v>469</v>
       </c>
-      <c r="M77" t="s">
-        <v>458</v>
+      <c r="L77" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="78" spans="1:13">
@@ -4219,8 +4042,11 @@
       <c r="K78">
         <v>470</v>
       </c>
+      <c r="L78" t="s">
+        <v>89</v>
+      </c>
       <c r="M78" t="s">
-        <v>459</v>
+        <v>304</v>
       </c>
     </row>
     <row r="79" spans="1:13">
@@ -4242,8 +4068,11 @@
       <c r="K79">
         <v>470</v>
       </c>
+      <c r="L79" t="s">
+        <v>90</v>
+      </c>
       <c r="M79" t="s">
-        <v>460</v>
+        <v>301</v>
       </c>
     </row>
     <row r="80" spans="1:13">
@@ -4265,8 +4094,11 @@
       <c r="K80">
         <v>470</v>
       </c>
+      <c r="L80" t="s">
+        <v>91</v>
+      </c>
       <c r="M80" t="s">
-        <v>461</v>
+        <v>311</v>
       </c>
     </row>
     <row r="81" spans="1:13">
@@ -4288,8 +4120,11 @@
       <c r="K81">
         <v>470</v>
       </c>
+      <c r="L81" t="s">
+        <v>92</v>
+      </c>
       <c r="M81" t="s">
-        <v>462</v>
+        <v>302</v>
       </c>
     </row>
     <row r="82" spans="1:13">
@@ -4311,8 +4146,11 @@
       <c r="K82">
         <v>470</v>
       </c>
+      <c r="L82" t="s">
+        <v>93</v>
+      </c>
       <c r="M82" t="s">
-        <v>463</v>
+        <v>304</v>
       </c>
     </row>
     <row r="83" spans="1:13">
@@ -4334,8 +4172,11 @@
       <c r="K83">
         <v>471</v>
       </c>
+      <c r="L83" t="s">
+        <v>94</v>
+      </c>
       <c r="M83" t="s">
-        <v>464</v>
+        <v>301</v>
       </c>
     </row>
     <row r="84" spans="1:13">
@@ -4357,8 +4198,11 @@
       <c r="K84">
         <v>470</v>
       </c>
+      <c r="L84" t="s">
+        <v>95</v>
+      </c>
       <c r="M84" t="s">
-        <v>465</v>
+        <v>302</v>
       </c>
     </row>
     <row r="85" spans="1:13">
@@ -4374,8 +4218,8 @@
       <c r="K85">
         <v>472</v>
       </c>
-      <c r="M85" t="s">
-        <v>466</v>
+      <c r="L85" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="86" spans="1:13">
@@ -4391,8 +4235,8 @@
       <c r="K86">
         <v>472</v>
       </c>
-      <c r="M86" t="s">
-        <v>467</v>
+      <c r="L86" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="87" spans="1:13">
@@ -4408,8 +4252,8 @@
       <c r="K87">
         <v>472</v>
       </c>
-      <c r="M87" t="s">
-        <v>468</v>
+      <c r="L87" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="88" spans="1:13">
@@ -4425,8 +4269,8 @@
       <c r="K88">
         <v>472</v>
       </c>
-      <c r="M88" t="s">
-        <v>469</v>
+      <c r="L88" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="89" spans="1:13">
@@ -4451,8 +4295,11 @@
       <c r="K89">
         <v>473</v>
       </c>
+      <c r="L89" t="s">
+        <v>100</v>
+      </c>
       <c r="M89" t="s">
-        <v>470</v>
+        <v>487</v>
       </c>
     </row>
     <row r="90" spans="1:13">
@@ -4477,8 +4324,11 @@
       <c r="K90">
         <v>473</v>
       </c>
+      <c r="L90" t="s">
+        <v>411</v>
+      </c>
       <c r="M90" t="s">
-        <v>471</v>
+        <v>488</v>
       </c>
     </row>
     <row r="91" spans="1:13">
@@ -4503,8 +4353,11 @@
       <c r="K91">
         <v>474</v>
       </c>
+      <c r="L91" t="s">
+        <v>102</v>
+      </c>
       <c r="M91" t="s">
-        <v>472</v>
+        <v>489</v>
       </c>
     </row>
     <row r="92" spans="1:13">
@@ -4529,8 +4382,11 @@
       <c r="K92">
         <v>473</v>
       </c>
+      <c r="L92" t="s">
+        <v>103</v>
+      </c>
       <c r="M92" t="s">
-        <v>473</v>
+        <v>490</v>
       </c>
     </row>
     <row r="93" spans="1:13">
@@ -4549,8 +4405,11 @@
       <c r="K93">
         <v>475</v>
       </c>
+      <c r="L93" t="s">
+        <v>104</v>
+      </c>
       <c r="M93" t="s">
-        <v>474</v>
+        <v>491</v>
       </c>
     </row>
     <row r="94" spans="1:13">
@@ -4569,8 +4428,11 @@
       <c r="K94">
         <v>475</v>
       </c>
+      <c r="L94" t="s">
+        <v>105</v>
+      </c>
       <c r="M94" t="s">
-        <v>475</v>
+        <v>491</v>
       </c>
     </row>
     <row r="95" spans="1:13">
@@ -4586,8 +4448,8 @@
       <c r="K95">
         <v>476</v>
       </c>
-      <c r="M95" t="s">
-        <v>476</v>
+      <c r="L95" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="96" spans="1:13">
@@ -4606,8 +4468,8 @@
       <c r="K96">
         <v>477</v>
       </c>
-      <c r="M96" t="s">
-        <v>477</v>
+      <c r="L96" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="97" spans="1:13">
@@ -4623,8 +4485,8 @@
       <c r="K97">
         <v>478</v>
       </c>
-      <c r="M97" t="s">
-        <v>478</v>
+      <c r="L97" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="98" spans="1:13">
@@ -4649,8 +4511,11 @@
       <c r="K98">
         <v>479</v>
       </c>
+      <c r="L98" t="s">
+        <v>412</v>
+      </c>
       <c r="M98" t="s">
-        <v>479</v>
+        <v>492</v>
       </c>
     </row>
     <row r="99" spans="1:13">
@@ -4672,8 +4537,11 @@
       <c r="K99">
         <v>480</v>
       </c>
+      <c r="L99" t="s">
+        <v>413</v>
+      </c>
       <c r="M99" t="s">
-        <v>480</v>
+        <v>321</v>
       </c>
     </row>
     <row r="100" spans="1:13">
@@ -4695,8 +4563,11 @@
       <c r="K100">
         <v>480</v>
       </c>
+      <c r="L100" t="s">
+        <v>414</v>
+      </c>
       <c r="M100" t="s">
-        <v>481</v>
+        <v>322</v>
       </c>
     </row>
     <row r="101" spans="1:13">
@@ -4718,8 +4589,11 @@
       <c r="K101">
         <v>480</v>
       </c>
+      <c r="L101" t="s">
+        <v>415</v>
+      </c>
       <c r="M101" t="s">
-        <v>482</v>
+        <v>321</v>
       </c>
     </row>
     <row r="102" spans="1:13">
@@ -4738,8 +4612,11 @@
       <c r="K102">
         <v>445</v>
       </c>
+      <c r="L102" t="s">
+        <v>113</v>
+      </c>
       <c r="M102" t="s">
-        <v>483</v>
+        <v>493</v>
       </c>
     </row>
     <row r="103" spans="1:13">
@@ -4761,8 +4638,11 @@
       <c r="K103">
         <v>481</v>
       </c>
+      <c r="L103" t="s">
+        <v>114</v>
+      </c>
       <c r="M103" t="s">
-        <v>484</v>
+        <v>493</v>
       </c>
     </row>
     <row r="104" spans="1:13">
@@ -4781,8 +4661,11 @@
       <c r="K104">
         <v>482</v>
       </c>
+      <c r="L104" t="s">
+        <v>115</v>
+      </c>
       <c r="M104" t="s">
-        <v>485</v>
+        <v>494</v>
       </c>
     </row>
     <row r="105" spans="1:13">
@@ -4798,8 +4681,8 @@
       <c r="K105">
         <v>483</v>
       </c>
-      <c r="M105" t="s">
-        <v>486</v>
+      <c r="L105" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="106" spans="1:13">
@@ -4818,8 +4701,8 @@
       <c r="K106">
         <v>455</v>
       </c>
-      <c r="M106" t="s">
-        <v>487</v>
+      <c r="L106" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="107" spans="1:13">
@@ -4841,8 +4724,11 @@
       <c r="K107">
         <v>484</v>
       </c>
+      <c r="L107" t="s">
+        <v>118</v>
+      </c>
       <c r="M107" t="s">
-        <v>488</v>
+        <v>495</v>
       </c>
     </row>
     <row r="108" spans="1:13">
@@ -4858,8 +4744,8 @@
       <c r="K108">
         <v>485</v>
       </c>
-      <c r="M108" t="s">
-        <v>489</v>
+      <c r="L108" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="109" spans="1:13">
@@ -4878,8 +4764,8 @@
       <c r="K109">
         <v>486</v>
       </c>
-      <c r="M109" t="s">
-        <v>490</v>
+      <c r="L109" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="110" spans="1:13">
@@ -4895,8 +4781,8 @@
       <c r="K110">
         <v>483</v>
       </c>
-      <c r="M110" t="s">
-        <v>491</v>
+      <c r="L110" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="111" spans="1:13">
@@ -4918,8 +4804,11 @@
       <c r="K111">
         <v>487</v>
       </c>
+      <c r="L111" t="s">
+        <v>122</v>
+      </c>
       <c r="M111" t="s">
-        <v>492</v>
+        <v>304</v>
       </c>
     </row>
     <row r="112" spans="1:13">
@@ -4941,8 +4830,11 @@
       <c r="K112">
         <v>487</v>
       </c>
+      <c r="L112" t="s">
+        <v>123</v>
+      </c>
       <c r="M112" t="s">
-        <v>493</v>
+        <v>304</v>
       </c>
     </row>
     <row r="113" spans="1:13">
@@ -4964,8 +4856,11 @@
       <c r="K113">
         <v>487</v>
       </c>
+      <c r="L113" t="s">
+        <v>124</v>
+      </c>
       <c r="M113" t="s">
-        <v>494</v>
+        <v>304</v>
       </c>
     </row>
     <row r="114" spans="1:13">
@@ -4987,8 +4882,11 @@
       <c r="K114">
         <v>487</v>
       </c>
+      <c r="L114" t="s">
+        <v>125</v>
+      </c>
       <c r="M114" t="s">
-        <v>495</v>
+        <v>304</v>
       </c>
     </row>
     <row r="115" spans="1:13">
@@ -5007,8 +4905,8 @@
       <c r="K115">
         <v>487</v>
       </c>
-      <c r="M115" t="s">
-        <v>496</v>
+      <c r="L115" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="116" spans="1:13">
@@ -5027,8 +4925,8 @@
       <c r="K116">
         <v>487</v>
       </c>
-      <c r="M116" t="s">
-        <v>497</v>
+      <c r="L116" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="117" spans="1:13">
@@ -5047,8 +4945,8 @@
       <c r="K117">
         <v>487</v>
       </c>
-      <c r="M117" t="s">
-        <v>498</v>
+      <c r="L117" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="118" spans="1:13">
@@ -5067,8 +4965,8 @@
       <c r="K118">
         <v>487</v>
       </c>
-      <c r="M118" t="s">
-        <v>499</v>
+      <c r="L118" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="119" spans="1:13">
@@ -5087,8 +4985,8 @@
       <c r="K119">
         <v>487</v>
       </c>
-      <c r="M119" t="s">
-        <v>500</v>
+      <c r="L119" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="120" spans="1:13">
@@ -5104,8 +5002,8 @@
       <c r="K120">
         <v>488</v>
       </c>
-      <c r="M120" t="s">
-        <v>501</v>
+      <c r="L120" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="121" spans="1:13">
@@ -5127,8 +5025,11 @@
       <c r="K121">
         <v>480</v>
       </c>
+      <c r="L121" t="s">
+        <v>416</v>
+      </c>
       <c r="M121" t="s">
-        <v>502</v>
+        <v>321</v>
       </c>
     </row>
     <row r="122" spans="1:13">
@@ -5147,8 +5048,11 @@
       <c r="K122">
         <v>489</v>
       </c>
+      <c r="L122" t="s">
+        <v>133</v>
+      </c>
       <c r="M122" t="s">
-        <v>503</v>
+        <v>449</v>
       </c>
     </row>
     <row r="123" spans="1:13">
@@ -5164,8 +5068,8 @@
       <c r="K123">
         <v>490</v>
       </c>
-      <c r="M123" t="s">
-        <v>504</v>
+      <c r="L123" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="124" spans="1:13">
@@ -5184,8 +5088,8 @@
       <c r="K124">
         <v>491</v>
       </c>
-      <c r="M124" t="s">
-        <v>505</v>
+      <c r="L124" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="125" spans="1:13">
@@ -5207,8 +5111,11 @@
       <c r="K125">
         <v>492</v>
       </c>
+      <c r="L125" t="s">
+        <v>417</v>
+      </c>
       <c r="M125" t="s">
-        <v>506</v>
+        <v>323</v>
       </c>
     </row>
     <row r="126" spans="1:13">
@@ -5230,8 +5137,11 @@
       <c r="K126">
         <v>480</v>
       </c>
+      <c r="L126" t="s">
+        <v>418</v>
+      </c>
       <c r="M126" t="s">
-        <v>507</v>
+        <v>322</v>
       </c>
     </row>
     <row r="127" spans="1:13">
@@ -5253,8 +5163,11 @@
       <c r="K127">
         <v>479</v>
       </c>
+      <c r="L127" t="s">
+        <v>419</v>
+      </c>
       <c r="M127" t="s">
-        <v>508</v>
+        <v>496</v>
       </c>
     </row>
     <row r="128" spans="1:13">
@@ -5276,8 +5189,11 @@
       <c r="K128">
         <v>479</v>
       </c>
+      <c r="L128" t="s">
+        <v>420</v>
+      </c>
       <c r="M128" t="s">
-        <v>509</v>
+        <v>497</v>
       </c>
     </row>
     <row r="129" spans="1:13">
@@ -5299,8 +5215,11 @@
       <c r="K129">
         <v>480</v>
       </c>
+      <c r="L129" t="s">
+        <v>421</v>
+      </c>
       <c r="M129" t="s">
-        <v>510</v>
+        <v>321</v>
       </c>
     </row>
     <row r="130" spans="1:13">
@@ -5325,8 +5244,11 @@
       <c r="K130">
         <v>443</v>
       </c>
+      <c r="L130" t="s">
+        <v>422</v>
+      </c>
       <c r="M130" t="s">
-        <v>511</v>
+        <v>483</v>
       </c>
     </row>
     <row r="131" spans="1:13">
@@ -5351,8 +5273,11 @@
       <c r="K131">
         <v>437</v>
       </c>
+      <c r="L131" t="s">
+        <v>423</v>
+      </c>
       <c r="M131" t="s">
-        <v>512</v>
+        <v>483</v>
       </c>
     </row>
     <row r="132" spans="1:13">
@@ -5371,8 +5296,11 @@
       <c r="K132">
         <v>493</v>
       </c>
+      <c r="L132" t="s">
+        <v>424</v>
+      </c>
       <c r="M132" t="s">
-        <v>513</v>
+        <v>317</v>
       </c>
     </row>
     <row r="133" spans="1:13">
@@ -5394,8 +5322,11 @@
       <c r="K133">
         <v>494</v>
       </c>
+      <c r="L133" t="s">
+        <v>144</v>
+      </c>
       <c r="M133" t="s">
-        <v>514</v>
+        <v>498</v>
       </c>
     </row>
     <row r="134" spans="1:13">
@@ -5417,8 +5348,11 @@
       <c r="K134">
         <v>494</v>
       </c>
+      <c r="L134" t="s">
+        <v>145</v>
+      </c>
       <c r="M134" t="s">
-        <v>515</v>
+        <v>499</v>
       </c>
     </row>
     <row r="135" spans="1:13">
@@ -5443,8 +5377,11 @@
       <c r="K135">
         <v>436</v>
       </c>
+      <c r="L135" t="s">
+        <v>146</v>
+      </c>
       <c r="M135" t="s">
-        <v>516</v>
+        <v>500</v>
       </c>
     </row>
     <row r="136" spans="1:13">
@@ -5469,8 +5406,11 @@
       <c r="K136">
         <v>436</v>
       </c>
+      <c r="L136" t="s">
+        <v>147</v>
+      </c>
       <c r="M136" t="s">
-        <v>517</v>
+        <v>501</v>
       </c>
     </row>
     <row r="137" spans="1:13">
@@ -5495,8 +5435,11 @@
       <c r="K137">
         <v>436</v>
       </c>
+      <c r="L137" t="s">
+        <v>148</v>
+      </c>
       <c r="M137" t="s">
-        <v>518</v>
+        <v>502</v>
       </c>
     </row>
     <row r="138" spans="1:13">
@@ -5521,8 +5464,11 @@
       <c r="K138">
         <v>436</v>
       </c>
+      <c r="L138" t="s">
+        <v>149</v>
+      </c>
       <c r="M138" t="s">
-        <v>519</v>
+        <v>503</v>
       </c>
     </row>
     <row r="139" spans="1:13">
@@ -5547,8 +5493,11 @@
       <c r="K139">
         <v>436</v>
       </c>
+      <c r="L139" t="s">
+        <v>150</v>
+      </c>
       <c r="M139" t="s">
-        <v>520</v>
+        <v>504</v>
       </c>
     </row>
     <row r="140" spans="1:13">
@@ -5573,8 +5522,11 @@
       <c r="K140">
         <v>436</v>
       </c>
+      <c r="L140" t="s">
+        <v>151</v>
+      </c>
       <c r="M140" t="s">
-        <v>521</v>
+        <v>505</v>
       </c>
     </row>
     <row r="141" spans="1:13">
@@ -5599,8 +5551,11 @@
       <c r="K141">
         <v>436</v>
       </c>
+      <c r="L141" t="s">
+        <v>152</v>
+      </c>
       <c r="M141" t="s">
-        <v>522</v>
+        <v>506</v>
       </c>
     </row>
     <row r="142" spans="1:13">
@@ -5622,8 +5577,11 @@
       <c r="K142">
         <v>436</v>
       </c>
+      <c r="L142" t="s">
+        <v>153</v>
+      </c>
       <c r="M142" t="s">
-        <v>523</v>
+        <v>507</v>
       </c>
     </row>
     <row r="143" spans="1:13">
@@ -5648,8 +5606,11 @@
       <c r="K143">
         <v>444</v>
       </c>
+      <c r="L143" t="s">
+        <v>154</v>
+      </c>
       <c r="M143" t="s">
-        <v>524</v>
+        <v>508</v>
       </c>
     </row>
     <row r="144" spans="1:13">
@@ -5674,8 +5635,11 @@
       <c r="K144">
         <v>436</v>
       </c>
+      <c r="L144" t="s">
+        <v>155</v>
+      </c>
       <c r="M144" t="s">
-        <v>525</v>
+        <v>509</v>
       </c>
     </row>
     <row r="145" spans="1:13">
@@ -5700,8 +5664,11 @@
       <c r="K145">
         <v>436</v>
       </c>
+      <c r="L145" t="s">
+        <v>156</v>
+      </c>
       <c r="M145" t="s">
-        <v>526</v>
+        <v>510</v>
       </c>
     </row>
     <row r="146" spans="1:13">
@@ -5726,8 +5693,11 @@
       <c r="K146">
         <v>444</v>
       </c>
+      <c r="L146" t="s">
+        <v>157</v>
+      </c>
       <c r="M146" t="s">
-        <v>527</v>
+        <v>511</v>
       </c>
     </row>
     <row r="147" spans="1:13">
@@ -5752,8 +5722,11 @@
       <c r="K147">
         <v>447</v>
       </c>
+      <c r="L147" t="s">
+        <v>425</v>
+      </c>
       <c r="M147" t="s">
-        <v>528</v>
+        <v>512</v>
       </c>
     </row>
     <row r="148" spans="1:13">
@@ -5775,8 +5748,11 @@
       <c r="K148">
         <v>495</v>
       </c>
+      <c r="L148" t="s">
+        <v>426</v>
+      </c>
       <c r="M148" t="s">
-        <v>529</v>
+        <v>513</v>
       </c>
     </row>
     <row r="149" spans="1:13">
@@ -5801,8 +5777,11 @@
       <c r="K149">
         <v>460</v>
       </c>
+      <c r="L149" t="s">
+        <v>160</v>
+      </c>
       <c r="M149" t="s">
-        <v>530</v>
+        <v>514</v>
       </c>
     </row>
     <row r="150" spans="1:13">
@@ -5824,8 +5803,11 @@
       <c r="K150">
         <v>439</v>
       </c>
+      <c r="L150" t="s">
+        <v>161</v>
+      </c>
       <c r="M150" t="s">
-        <v>531</v>
+        <v>446</v>
       </c>
     </row>
     <row r="151" spans="1:13">
@@ -5847,8 +5829,11 @@
       <c r="K151">
         <v>439</v>
       </c>
+      <c r="L151" t="s">
+        <v>162</v>
+      </c>
       <c r="M151" t="s">
-        <v>532</v>
+        <v>446</v>
       </c>
     </row>
     <row r="152" spans="1:13">
@@ -5867,8 +5852,8 @@
       <c r="K152">
         <v>486</v>
       </c>
-      <c r="M152" t="s">
-        <v>533</v>
+      <c r="L152" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="153" spans="1:13">
@@ -5884,8 +5869,8 @@
       <c r="K153">
         <v>496</v>
       </c>
-      <c r="M153" t="s">
-        <v>534</v>
+      <c r="L153" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="154" spans="1:13">
@@ -5901,8 +5886,8 @@
       <c r="K154">
         <v>497</v>
       </c>
-      <c r="M154" t="s">
-        <v>535</v>
+      <c r="L154" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="155" spans="1:13">
@@ -5921,8 +5906,8 @@
       <c r="K155">
         <v>498</v>
       </c>
-      <c r="M155" t="s">
-        <v>536</v>
+      <c r="L155" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="156" spans="1:13">
@@ -5941,8 +5926,8 @@
       <c r="K156">
         <v>498</v>
       </c>
-      <c r="M156" t="s">
-        <v>537</v>
+      <c r="L156" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="157" spans="1:13">
@@ -5961,8 +5946,8 @@
       <c r="K157">
         <v>498</v>
       </c>
-      <c r="M157" t="s">
-        <v>538</v>
+      <c r="L157" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="158" spans="1:13">
@@ -5981,8 +5966,8 @@
       <c r="K158">
         <v>498</v>
       </c>
-      <c r="M158" t="s">
-        <v>539</v>
+      <c r="L158" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="159" spans="1:13">
@@ -6001,8 +5986,11 @@
       <c r="K159">
         <v>441</v>
       </c>
+      <c r="L159" t="s">
+        <v>170</v>
+      </c>
       <c r="M159" t="s">
-        <v>540</v>
+        <v>515</v>
       </c>
     </row>
     <row r="160" spans="1:13">
@@ -6021,8 +6009,11 @@
       <c r="K160">
         <v>441</v>
       </c>
+      <c r="L160" t="s">
+        <v>171</v>
+      </c>
       <c r="M160" t="s">
-        <v>541</v>
+        <v>516</v>
       </c>
     </row>
     <row r="161" spans="1:13">
@@ -6041,8 +6032,11 @@
       <c r="K161">
         <v>441</v>
       </c>
+      <c r="L161" t="s">
+        <v>172</v>
+      </c>
       <c r="M161" t="s">
-        <v>542</v>
+        <v>448</v>
       </c>
     </row>
     <row r="162" spans="1:13">
@@ -6061,8 +6055,11 @@
       <c r="K162">
         <v>441</v>
       </c>
+      <c r="L162" t="s">
+        <v>173</v>
+      </c>
       <c r="M162" t="s">
-        <v>543</v>
+        <v>491</v>
       </c>
     </row>
     <row r="163" spans="1:13">
@@ -6081,8 +6078,11 @@
       <c r="K163">
         <v>499</v>
       </c>
+      <c r="L163" t="s">
+        <v>174</v>
+      </c>
       <c r="M163" t="s">
-        <v>544</v>
+        <v>517</v>
       </c>
     </row>
     <row r="164" spans="1:13">
@@ -6101,8 +6101,11 @@
       <c r="K164">
         <v>499</v>
       </c>
+      <c r="L164" t="s">
+        <v>175</v>
+      </c>
       <c r="M164" t="s">
-        <v>545</v>
+        <v>452</v>
       </c>
     </row>
     <row r="165" spans="1:13">
@@ -6121,8 +6124,11 @@
       <c r="K165">
         <v>499</v>
       </c>
+      <c r="L165" t="s">
+        <v>176</v>
+      </c>
       <c r="M165" t="s">
-        <v>546</v>
+        <v>518</v>
       </c>
     </row>
     <row r="166" spans="1:13">
@@ -6141,8 +6147,11 @@
       <c r="K166">
         <v>442</v>
       </c>
+      <c r="L166" t="s">
+        <v>177</v>
+      </c>
       <c r="M166" t="s">
-        <v>547</v>
+        <v>498</v>
       </c>
     </row>
     <row r="167" spans="1:13">
@@ -6161,8 +6170,11 @@
       <c r="K167">
         <v>442</v>
       </c>
+      <c r="L167" t="s">
+        <v>178</v>
+      </c>
       <c r="M167" t="s">
-        <v>548</v>
+        <v>498</v>
       </c>
     </row>
     <row r="168" spans="1:13">
@@ -6181,8 +6193,11 @@
       <c r="K168">
         <v>500</v>
       </c>
+      <c r="L168" t="s">
+        <v>179</v>
+      </c>
       <c r="M168" t="s">
-        <v>549</v>
+        <v>452</v>
       </c>
     </row>
     <row r="169" spans="1:13">
@@ -6204,8 +6219,11 @@
       <c r="K169">
         <v>501</v>
       </c>
+      <c r="L169" t="s">
+        <v>180</v>
+      </c>
       <c r="M169" t="s">
-        <v>550</v>
+        <v>491</v>
       </c>
     </row>
     <row r="170" spans="1:13">
@@ -6224,8 +6242,11 @@
       <c r="K170">
         <v>501</v>
       </c>
+      <c r="L170" t="s">
+        <v>181</v>
+      </c>
       <c r="M170" t="s">
-        <v>551</v>
+        <v>519</v>
       </c>
     </row>
     <row r="171" spans="1:13">
@@ -6244,8 +6265,11 @@
       <c r="K171">
         <v>490</v>
       </c>
+      <c r="L171" t="s">
+        <v>182</v>
+      </c>
       <c r="M171" t="s">
-        <v>552</v>
+        <v>498</v>
       </c>
     </row>
     <row r="172" spans="1:13">
@@ -6267,8 +6291,11 @@
       <c r="K172">
         <v>439</v>
       </c>
+      <c r="L172" t="s">
+        <v>183</v>
+      </c>
       <c r="M172" t="s">
-        <v>553</v>
+        <v>469</v>
       </c>
     </row>
     <row r="173" spans="1:13">
@@ -6287,8 +6314,11 @@
       <c r="K173">
         <v>499</v>
       </c>
+      <c r="L173" t="s">
+        <v>184</v>
+      </c>
       <c r="M173" t="s">
-        <v>554</v>
+        <v>515</v>
       </c>
     </row>
     <row r="174" spans="1:13">
@@ -6307,8 +6337,11 @@
       <c r="K174">
         <v>502</v>
       </c>
+      <c r="L174" t="s">
+        <v>185</v>
+      </c>
       <c r="M174" t="s">
-        <v>555</v>
+        <v>520</v>
       </c>
     </row>
     <row r="175" spans="1:13">
@@ -6330,8 +6363,11 @@
       <c r="K175">
         <v>502</v>
       </c>
+      <c r="L175" t="s">
+        <v>186</v>
+      </c>
       <c r="M175" t="s">
-        <v>556</v>
+        <v>521</v>
       </c>
     </row>
     <row r="176" spans="1:13">
@@ -6350,8 +6386,11 @@
       <c r="K176">
         <v>503</v>
       </c>
+      <c r="L176" t="s">
+        <v>187</v>
+      </c>
       <c r="M176" t="s">
-        <v>557</v>
+        <v>453</v>
       </c>
     </row>
     <row r="177" spans="1:13">
@@ -6373,8 +6412,11 @@
       <c r="K177">
         <v>504</v>
       </c>
+      <c r="L177" t="s">
+        <v>188</v>
+      </c>
       <c r="M177" t="s">
-        <v>558</v>
+        <v>484</v>
       </c>
     </row>
     <row r="178" spans="1:13">
@@ -6396,8 +6438,11 @@
       <c r="K178">
         <v>439</v>
       </c>
+      <c r="L178" t="s">
+        <v>189</v>
+      </c>
       <c r="M178" t="s">
-        <v>559</v>
+        <v>482</v>
       </c>
     </row>
     <row r="179" spans="1:13">
@@ -6413,8 +6458,8 @@
       <c r="K179">
         <v>505</v>
       </c>
-      <c r="M179" t="s">
-        <v>560</v>
+      <c r="L179" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="180" spans="1:13">
@@ -6436,8 +6481,11 @@
       <c r="K180">
         <v>494</v>
       </c>
+      <c r="L180" t="s">
+        <v>191</v>
+      </c>
       <c r="M180" t="s">
-        <v>561</v>
+        <v>522</v>
       </c>
     </row>
     <row r="181" spans="1:13">
@@ -6459,8 +6507,11 @@
       <c r="K181">
         <v>494</v>
       </c>
+      <c r="L181" t="s">
+        <v>192</v>
+      </c>
       <c r="M181" t="s">
-        <v>562</v>
+        <v>522</v>
       </c>
     </row>
     <row r="182" spans="1:13">
@@ -6482,8 +6533,11 @@
       <c r="K182">
         <v>470</v>
       </c>
+      <c r="L182" t="s">
+        <v>193</v>
+      </c>
       <c r="M182" t="s">
-        <v>563</v>
+        <v>301</v>
       </c>
     </row>
     <row r="183" spans="1:13">
@@ -6505,8 +6559,11 @@
       <c r="K183">
         <v>470</v>
       </c>
+      <c r="L183" t="s">
+        <v>194</v>
+      </c>
       <c r="M183" t="s">
-        <v>564</v>
+        <v>304</v>
       </c>
     </row>
     <row r="184" spans="1:13">
@@ -6528,8 +6585,11 @@
       <c r="K184">
         <v>439</v>
       </c>
+      <c r="L184" t="s">
+        <v>195</v>
+      </c>
       <c r="M184" t="s">
-        <v>565</v>
+        <v>516</v>
       </c>
     </row>
     <row r="185" spans="1:13">
@@ -6551,8 +6611,11 @@
       <c r="K185">
         <v>439</v>
       </c>
+      <c r="L185" t="s">
+        <v>196</v>
+      </c>
       <c r="M185" t="s">
-        <v>566</v>
+        <v>516</v>
       </c>
     </row>
     <row r="186" spans="1:13">
@@ -6571,8 +6634,8 @@
       <c r="K186">
         <v>506</v>
       </c>
-      <c r="M186" t="s">
-        <v>567</v>
+      <c r="L186" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="187" spans="1:13">
@@ -6591,8 +6654,8 @@
       <c r="K187">
         <v>506</v>
       </c>
-      <c r="M187" t="s">
-        <v>568</v>
+      <c r="L187" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="188" spans="1:13">
@@ -6614,8 +6677,11 @@
       <c r="K188">
         <v>470</v>
       </c>
+      <c r="L188" t="s">
+        <v>199</v>
+      </c>
       <c r="M188" t="s">
-        <v>569</v>
+        <v>302</v>
       </c>
     </row>
     <row r="189" spans="1:13">
@@ -6637,8 +6703,11 @@
       <c r="K189">
         <v>470</v>
       </c>
+      <c r="L189" t="s">
+        <v>200</v>
+      </c>
       <c r="M189" t="s">
-        <v>570</v>
+        <v>301</v>
       </c>
     </row>
     <row r="190" spans="1:13">
@@ -6660,8 +6729,11 @@
       <c r="K190">
         <v>470</v>
       </c>
+      <c r="L190" t="s">
+        <v>201</v>
+      </c>
       <c r="M190" t="s">
-        <v>571</v>
+        <v>304</v>
       </c>
     </row>
     <row r="191" spans="1:13">
@@ -6680,8 +6752,11 @@
       <c r="K191">
         <v>465</v>
       </c>
+      <c r="L191" t="s">
+        <v>202</v>
+      </c>
       <c r="M191" t="s">
-        <v>572</v>
+        <v>523</v>
       </c>
     </row>
     <row r="192" spans="1:13">
@@ -6700,8 +6775,11 @@
       <c r="K192">
         <v>465</v>
       </c>
+      <c r="L192" t="s">
+        <v>203</v>
+      </c>
       <c r="M192" t="s">
-        <v>573</v>
+        <v>523</v>
       </c>
     </row>
     <row r="193" spans="1:13">
@@ -6720,8 +6798,11 @@
       <c r="K193">
         <v>465</v>
       </c>
+      <c r="L193" t="s">
+        <v>204</v>
+      </c>
       <c r="M193" t="s">
-        <v>574</v>
+        <v>523</v>
       </c>
     </row>
     <row r="194" spans="1:13">
@@ -6740,8 +6821,11 @@
       <c r="K194">
         <v>465</v>
       </c>
+      <c r="L194" t="s">
+        <v>205</v>
+      </c>
       <c r="M194" t="s">
-        <v>575</v>
+        <v>519</v>
       </c>
     </row>
     <row r="195" spans="1:13">
@@ -6766,8 +6850,11 @@
       <c r="K195">
         <v>436</v>
       </c>
+      <c r="L195" t="s">
+        <v>206</v>
+      </c>
       <c r="M195" t="s">
-        <v>576</v>
+        <v>524</v>
       </c>
     </row>
     <row r="196" spans="1:13">
@@ -6792,8 +6879,11 @@
       <c r="K196">
         <v>444</v>
       </c>
+      <c r="L196" t="s">
+        <v>207</v>
+      </c>
       <c r="M196" t="s">
-        <v>577</v>
+        <v>525</v>
       </c>
     </row>
     <row r="197" spans="1:13">
@@ -6818,8 +6908,11 @@
       <c r="K197">
         <v>444</v>
       </c>
+      <c r="L197" t="s">
+        <v>208</v>
+      </c>
       <c r="M197" t="s">
-        <v>578</v>
+        <v>509</v>
       </c>
     </row>
     <row r="198" spans="1:13">
@@ -6844,8 +6937,11 @@
       <c r="K198">
         <v>444</v>
       </c>
+      <c r="L198" t="s">
+        <v>209</v>
+      </c>
       <c r="M198" t="s">
-        <v>579</v>
+        <v>526</v>
       </c>
     </row>
     <row r="199" spans="1:13">
@@ -6861,8 +6957,8 @@
       <c r="K199">
         <v>507</v>
       </c>
-      <c r="M199" t="s">
-        <v>580</v>
+      <c r="L199" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="200" spans="1:13">
@@ -6884,8 +6980,11 @@
       <c r="K200">
         <v>508</v>
       </c>
+      <c r="L200" t="s">
+        <v>427</v>
+      </c>
       <c r="M200" t="s">
-        <v>581</v>
+        <v>457</v>
       </c>
     </row>
     <row r="201" spans="1:13">
@@ -6907,8 +7006,11 @@
       <c r="K201">
         <v>449</v>
       </c>
+      <c r="L201" t="s">
+        <v>428</v>
+      </c>
       <c r="M201" t="s">
-        <v>582</v>
+        <v>456</v>
       </c>
     </row>
     <row r="202" spans="1:13">
@@ -6927,8 +7029,11 @@
       <c r="K202">
         <v>508</v>
       </c>
+      <c r="L202" t="s">
+        <v>429</v>
+      </c>
       <c r="M202" t="s">
-        <v>583</v>
+        <v>299</v>
       </c>
     </row>
     <row r="203" spans="1:13">
@@ -6944,8 +7049,8 @@
       <c r="K203">
         <v>509</v>
       </c>
-      <c r="M203" t="s">
-        <v>584</v>
+      <c r="L203" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="204" spans="1:13">
@@ -6964,8 +7069,11 @@
       <c r="K204">
         <v>510</v>
       </c>
+      <c r="L204" t="s">
+        <v>215</v>
+      </c>
       <c r="M204" t="s">
-        <v>585</v>
+        <v>301</v>
       </c>
     </row>
     <row r="205" spans="1:13">
@@ -6984,8 +7092,11 @@
       <c r="K205">
         <v>510</v>
       </c>
+      <c r="L205" t="s">
+        <v>216</v>
+      </c>
       <c r="M205" t="s">
-        <v>586</v>
+        <v>304</v>
       </c>
     </row>
     <row r="206" spans="1:13">
@@ -7004,8 +7115,11 @@
       <c r="K206">
         <v>510</v>
       </c>
+      <c r="L206" t="s">
+        <v>217</v>
+      </c>
       <c r="M206" t="s">
-        <v>587</v>
+        <v>304</v>
       </c>
     </row>
     <row r="207" spans="1:13">
@@ -7021,8 +7135,8 @@
       <c r="K207">
         <v>510</v>
       </c>
-      <c r="M207" t="s">
-        <v>588</v>
+      <c r="L207" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="208" spans="1:13">
@@ -7041,8 +7155,11 @@
       <c r="K208">
         <v>503</v>
       </c>
+      <c r="L208" t="s">
+        <v>219</v>
+      </c>
       <c r="M208" t="s">
-        <v>589</v>
+        <v>527</v>
       </c>
     </row>
     <row r="209" spans="1:13">
@@ -7061,8 +7178,11 @@
       <c r="K209">
         <v>503</v>
       </c>
+      <c r="L209" t="s">
+        <v>220</v>
+      </c>
       <c r="M209" t="s">
-        <v>590</v>
+        <v>527</v>
       </c>
     </row>
     <row r="210" spans="1:13">
@@ -7081,8 +7201,11 @@
       <c r="K210">
         <v>511</v>
       </c>
+      <c r="L210" t="s">
+        <v>221</v>
+      </c>
       <c r="M210" t="s">
-        <v>591</v>
+        <v>528</v>
       </c>
     </row>
     <row r="211" spans="1:13">
@@ -7101,8 +7224,11 @@
       <c r="K211">
         <v>511</v>
       </c>
+      <c r="L211" t="s">
+        <v>222</v>
+      </c>
       <c r="M211" t="s">
-        <v>592</v>
+        <v>528</v>
       </c>
     </row>
     <row r="212" spans="1:13">
@@ -7121,8 +7247,11 @@
       <c r="K212">
         <v>511</v>
       </c>
+      <c r="L212" t="s">
+        <v>223</v>
+      </c>
       <c r="M212" t="s">
-        <v>593</v>
+        <v>528</v>
       </c>
     </row>
     <row r="213" spans="1:13">
@@ -7141,8 +7270,11 @@
       <c r="K213">
         <v>512</v>
       </c>
+      <c r="L213" t="s">
+        <v>224</v>
+      </c>
       <c r="M213" t="s">
-        <v>594</v>
+        <v>528</v>
       </c>
     </row>
     <row r="214" spans="1:13">
@@ -7161,8 +7293,11 @@
       <c r="K214">
         <v>512</v>
       </c>
+      <c r="L214" t="s">
+        <v>225</v>
+      </c>
       <c r="M214" t="s">
-        <v>595</v>
+        <v>528</v>
       </c>
     </row>
     <row r="215" spans="1:13">
@@ -7181,8 +7316,11 @@
       <c r="K215">
         <v>511</v>
       </c>
+      <c r="L215" t="s">
+        <v>226</v>
+      </c>
       <c r="M215" t="s">
-        <v>596</v>
+        <v>528</v>
       </c>
     </row>
     <row r="216" spans="1:13">
@@ -7204,8 +7342,11 @@
       <c r="K216">
         <v>513</v>
       </c>
+      <c r="L216" t="s">
+        <v>227</v>
+      </c>
       <c r="M216" t="s">
-        <v>597</v>
+        <v>529</v>
       </c>
     </row>
     <row r="217" spans="1:13">
@@ -7230,8 +7371,11 @@
       <c r="K217">
         <v>466</v>
       </c>
+      <c r="L217" t="s">
+        <v>228</v>
+      </c>
       <c r="M217" t="s">
-        <v>598</v>
+        <v>486</v>
       </c>
     </row>
     <row r="218" spans="1:13">
@@ -7256,8 +7400,11 @@
       <c r="K218">
         <v>466</v>
       </c>
+      <c r="L218" t="s">
+        <v>229</v>
+      </c>
       <c r="M218" t="s">
-        <v>599</v>
+        <v>486</v>
       </c>
     </row>
     <row r="219" spans="1:13">
@@ -7276,8 +7423,11 @@
       <c r="K219">
         <v>514</v>
       </c>
+      <c r="L219" t="s">
+        <v>230</v>
+      </c>
       <c r="M219" t="s">
-        <v>600</v>
+        <v>301</v>
       </c>
     </row>
     <row r="220" spans="1:13">
@@ -7296,8 +7446,11 @@
       <c r="K220">
         <v>515</v>
       </c>
+      <c r="L220" t="s">
+        <v>430</v>
+      </c>
       <c r="M220" t="s">
-        <v>601</v>
+        <v>306</v>
       </c>
     </row>
     <row r="221" spans="1:13">
@@ -7316,8 +7469,11 @@
       <c r="K221">
         <v>457</v>
       </c>
+      <c r="L221" t="s">
+        <v>431</v>
+      </c>
       <c r="M221" t="s">
-        <v>602</v>
+        <v>307</v>
       </c>
     </row>
     <row r="222" spans="1:13">
@@ -7336,8 +7492,8 @@
       <c r="K222">
         <v>516</v>
       </c>
-      <c r="M222" t="s">
-        <v>603</v>
+      <c r="L222" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="223" spans="1:13">
@@ -7353,8 +7509,8 @@
       <c r="K223">
         <v>517</v>
       </c>
-      <c r="M223" t="s">
-        <v>604</v>
+      <c r="L223" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="224" spans="1:13">
@@ -7370,8 +7526,8 @@
       <c r="K224">
         <v>518</v>
       </c>
-      <c r="M224" t="s">
-        <v>605</v>
+      <c r="L224" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="225" spans="1:13">
@@ -7387,8 +7543,8 @@
       <c r="K225">
         <v>518</v>
       </c>
-      <c r="M225" t="s">
-        <v>606</v>
+      <c r="L225" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="226" spans="1:13">
@@ -7404,8 +7560,8 @@
       <c r="K226">
         <v>519</v>
       </c>
-      <c r="M226" t="s">
-        <v>607</v>
+      <c r="L226" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="227" spans="1:13">
@@ -7421,8 +7577,8 @@
       <c r="K227">
         <v>519</v>
       </c>
-      <c r="M227" t="s">
-        <v>608</v>
+      <c r="L227" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="228" spans="1:13">
@@ -7438,8 +7594,8 @@
       <c r="K228">
         <v>519</v>
       </c>
-      <c r="M228" t="s">
-        <v>609</v>
+      <c r="L228" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="229" spans="1:13">
@@ -7455,8 +7611,8 @@
       <c r="K229">
         <v>520</v>
       </c>
-      <c r="M229" t="s">
-        <v>610</v>
+      <c r="L229" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="230" spans="1:13">
@@ -7475,8 +7631,11 @@
       <c r="K230">
         <v>521</v>
       </c>
+      <c r="L230" t="s">
+        <v>241</v>
+      </c>
       <c r="M230" t="s">
-        <v>611</v>
+        <v>530</v>
       </c>
     </row>
     <row r="231" spans="1:13">
@@ -7495,8 +7654,11 @@
       <c r="K231">
         <v>522</v>
       </c>
+      <c r="L231" t="s">
+        <v>242</v>
+      </c>
       <c r="M231" t="s">
-        <v>612</v>
+        <v>531</v>
       </c>
     </row>
     <row r="232" spans="1:13">
@@ -7515,8 +7677,11 @@
       <c r="K232">
         <v>522</v>
       </c>
+      <c r="L232" t="s">
+        <v>243</v>
+      </c>
       <c r="M232" t="s">
-        <v>613</v>
+        <v>531</v>
       </c>
     </row>
     <row r="233" spans="1:13">
@@ -7535,8 +7700,11 @@
       <c r="K233">
         <v>522</v>
       </c>
+      <c r="L233" t="s">
+        <v>244</v>
+      </c>
       <c r="M233" t="s">
-        <v>614</v>
+        <v>531</v>
       </c>
     </row>
     <row r="234" spans="1:13">
@@ -7555,8 +7723,11 @@
       <c r="K234">
         <v>499</v>
       </c>
+      <c r="L234" t="s">
+        <v>245</v>
+      </c>
       <c r="M234" t="s">
-        <v>615</v>
+        <v>449</v>
       </c>
     </row>
     <row r="235" spans="1:13">
@@ -7575,8 +7746,11 @@
       <c r="K235">
         <v>490</v>
       </c>
+      <c r="L235" t="s">
+        <v>246</v>
+      </c>
       <c r="M235" t="s">
-        <v>616</v>
+        <v>498</v>
       </c>
     </row>
     <row r="236" spans="1:13">
@@ -7595,8 +7769,11 @@
       <c r="K236">
         <v>490</v>
       </c>
+      <c r="L236" t="s">
+        <v>247</v>
+      </c>
       <c r="M236" t="s">
-        <v>617</v>
+        <v>498</v>
       </c>
     </row>
     <row r="237" spans="1:13">
@@ -7615,8 +7792,11 @@
       <c r="K237">
         <v>499</v>
       </c>
+      <c r="L237" t="s">
+        <v>248</v>
+      </c>
       <c r="M237" t="s">
-        <v>618</v>
+        <v>532</v>
       </c>
     </row>
     <row r="238" spans="1:13">
@@ -7635,8 +7815,11 @@
       <c r="K238">
         <v>499</v>
       </c>
+      <c r="L238" t="s">
+        <v>249</v>
+      </c>
       <c r="M238" t="s">
-        <v>619</v>
+        <v>498</v>
       </c>
     </row>
     <row r="239" spans="1:13">
@@ -7655,8 +7838,11 @@
       <c r="K239">
         <v>523</v>
       </c>
+      <c r="L239" t="s">
+        <v>250</v>
+      </c>
       <c r="M239" t="s">
-        <v>620</v>
+        <v>452</v>
       </c>
     </row>
     <row r="240" spans="1:13">
@@ -7678,8 +7864,11 @@
       <c r="K240">
         <v>447</v>
       </c>
+      <c r="L240" t="s">
+        <v>432</v>
+      </c>
       <c r="M240" t="s">
-        <v>621</v>
+        <v>533</v>
       </c>
     </row>
     <row r="241" spans="1:13">
@@ -7695,8 +7884,8 @@
       <c r="K241">
         <v>517</v>
       </c>
-      <c r="M241" t="s">
-        <v>622</v>
+      <c r="L241" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="242" spans="1:13">
@@ -7712,8 +7901,8 @@
       <c r="K242">
         <v>524</v>
       </c>
-      <c r="M242" t="s">
-        <v>623</v>
+      <c r="L242" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="243" spans="1:13">
@@ -7729,8 +7918,8 @@
       <c r="K243">
         <v>524</v>
       </c>
-      <c r="M243" t="s">
-        <v>624</v>
+      <c r="L243" t="s">
+        <v>254</v>
       </c>
     </row>
     <row r="244" spans="1:13">
@@ -7746,8 +7935,8 @@
       <c r="K244">
         <v>518</v>
       </c>
-      <c r="M244" t="s">
-        <v>625</v>
+      <c r="L244" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="245" spans="1:13">
@@ -7763,8 +7952,8 @@
       <c r="K245">
         <v>517</v>
       </c>
-      <c r="M245" t="s">
-        <v>626</v>
+      <c r="L245" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="246" spans="1:13">
@@ -7783,8 +7972,11 @@
       <c r="K246">
         <v>525</v>
       </c>
+      <c r="L246" t="s">
+        <v>257</v>
+      </c>
       <c r="M246" t="s">
-        <v>627</v>
+        <v>302</v>
       </c>
     </row>
     <row r="247" spans="1:13">
@@ -7803,8 +7995,11 @@
       <c r="K247">
         <v>525</v>
       </c>
+      <c r="L247" t="s">
+        <v>258</v>
+      </c>
       <c r="M247" t="s">
-        <v>628</v>
+        <v>302</v>
       </c>
     </row>
     <row r="248" spans="1:13">
@@ -7826,8 +8021,11 @@
       <c r="K248">
         <v>526</v>
       </c>
+      <c r="L248" t="s">
+        <v>259</v>
+      </c>
       <c r="M248" t="s">
-        <v>629</v>
+        <v>447</v>
       </c>
     </row>
     <row r="249" spans="1:13">
@@ -7846,8 +8044,11 @@
       <c r="K249">
         <v>526</v>
       </c>
+      <c r="L249" t="s">
+        <v>260</v>
+      </c>
       <c r="M249" t="s">
-        <v>630</v>
+        <v>452</v>
       </c>
     </row>
     <row r="250" spans="1:13">
@@ -7869,8 +8070,11 @@
       <c r="K250">
         <v>526</v>
       </c>
+      <c r="L250" t="s">
+        <v>261</v>
+      </c>
       <c r="M250" t="s">
-        <v>631</v>
+        <v>452</v>
       </c>
     </row>
     <row r="251" spans="1:13">
@@ -7889,8 +8093,11 @@
       <c r="K251">
         <v>500</v>
       </c>
+      <c r="L251" t="s">
+        <v>262</v>
+      </c>
       <c r="M251" t="s">
-        <v>632</v>
+        <v>498</v>
       </c>
     </row>
     <row r="252" spans="1:13">
@@ -7912,8 +8119,11 @@
       <c r="K252">
         <v>527</v>
       </c>
+      <c r="L252" t="s">
+        <v>263</v>
+      </c>
       <c r="M252" t="s">
-        <v>633</v>
+        <v>534</v>
       </c>
     </row>
     <row r="253" spans="1:13">
@@ -7929,8 +8139,8 @@
       <c r="K253">
         <v>528</v>
       </c>
-      <c r="M253" t="s">
-        <v>634</v>
+      <c r="L253" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="254" spans="1:13">
@@ -7946,8 +8156,8 @@
       <c r="K254">
         <v>517</v>
       </c>
-      <c r="M254" t="s">
-        <v>635</v>
+      <c r="L254" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="255" spans="1:13">
@@ -7963,8 +8173,8 @@
       <c r="K255">
         <v>524</v>
       </c>
-      <c r="M255" t="s">
-        <v>636</v>
+      <c r="L255" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="256" spans="1:13">
@@ -7980,8 +8190,8 @@
       <c r="K256">
         <v>529</v>
       </c>
-      <c r="M256" t="s">
-        <v>637</v>
+      <c r="L256" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="257" spans="1:13">
@@ -7997,8 +8207,8 @@
       <c r="K257">
         <v>529</v>
       </c>
-      <c r="M257" t="s">
-        <v>638</v>
+      <c r="L257" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="258" spans="1:13">
@@ -8017,8 +8227,11 @@
       <c r="K258">
         <v>499</v>
       </c>
+      <c r="L258" t="s">
+        <v>269</v>
+      </c>
       <c r="M258" t="s">
-        <v>639</v>
+        <v>535</v>
       </c>
     </row>
     <row r="259" spans="1:13">
@@ -8037,8 +8250,11 @@
       <c r="K259">
         <v>499</v>
       </c>
+      <c r="L259" t="s">
+        <v>270</v>
+      </c>
       <c r="M259" t="s">
-        <v>640</v>
+        <v>520</v>
       </c>
     </row>
     <row r="260" spans="1:13">
@@ -8057,8 +8273,11 @@
       <c r="K260">
         <v>499</v>
       </c>
+      <c r="L260" t="s">
+        <v>271</v>
+      </c>
       <c r="M260" t="s">
-        <v>641</v>
+        <v>532</v>
       </c>
     </row>
     <row r="261" spans="1:13">
@@ -8077,8 +8296,11 @@
       <c r="K261">
         <v>490</v>
       </c>
+      <c r="L261" t="s">
+        <v>272</v>
+      </c>
       <c r="M261" t="s">
-        <v>642</v>
+        <v>498</v>
       </c>
     </row>
     <row r="262" spans="1:13">
@@ -8097,8 +8319,11 @@
       <c r="K262">
         <v>490</v>
       </c>
+      <c r="L262" t="s">
+        <v>273</v>
+      </c>
       <c r="M262" t="s">
-        <v>643</v>
+        <v>498</v>
       </c>
     </row>
     <row r="263" spans="1:13">
@@ -8117,8 +8342,11 @@
       <c r="K263">
         <v>499</v>
       </c>
+      <c r="L263" t="s">
+        <v>274</v>
+      </c>
       <c r="M263" t="s">
-        <v>644</v>
+        <v>536</v>
       </c>
     </row>
     <row r="264" spans="1:13">
@@ -8137,8 +8365,11 @@
       <c r="K264">
         <v>490</v>
       </c>
+      <c r="L264" t="s">
+        <v>275</v>
+      </c>
       <c r="M264" t="s">
-        <v>645</v>
+        <v>498</v>
       </c>
     </row>
     <row r="265" spans="1:13">
@@ -8157,8 +8388,11 @@
       <c r="K265">
         <v>530</v>
       </c>
+      <c r="L265" t="s">
+        <v>276</v>
+      </c>
       <c r="M265" t="s">
-        <v>646</v>
+        <v>498</v>
       </c>
     </row>
     <row r="266" spans="1:13">
@@ -8177,8 +8411,11 @@
       <c r="K266">
         <v>531</v>
       </c>
+      <c r="L266" t="s">
+        <v>277</v>
+      </c>
       <c r="M266" t="s">
-        <v>647</v>
+        <v>453</v>
       </c>
     </row>
     <row r="267" spans="1:13">
@@ -8197,8 +8434,11 @@
       <c r="K267">
         <v>532</v>
       </c>
+      <c r="L267" t="s">
+        <v>278</v>
+      </c>
       <c r="M267" t="s">
-        <v>648</v>
+        <v>314</v>
       </c>
     </row>
     <row r="268" spans="1:13">
@@ -8214,8 +8454,8 @@
       <c r="K268">
         <v>533</v>
       </c>
-      <c r="M268" t="s">
-        <v>649</v>
+      <c r="L268" t="s">
+        <v>279</v>
       </c>
     </row>
     <row r="269" spans="1:13">
@@ -8240,8 +8480,11 @@
       <c r="K269">
         <v>466</v>
       </c>
+      <c r="L269" t="s">
+        <v>280</v>
+      </c>
       <c r="M269" t="s">
-        <v>650</v>
+        <v>486</v>
       </c>
     </row>
     <row r="270" spans="1:13">
@@ -8260,8 +8503,11 @@
       <c r="K270">
         <v>512</v>
       </c>
+      <c r="L270" t="s">
+        <v>281</v>
+      </c>
       <c r="M270" t="s">
-        <v>651</v>
+        <v>528</v>
       </c>
     </row>
     <row r="271" spans="1:13">
@@ -8280,8 +8526,11 @@
       <c r="K271">
         <v>534</v>
       </c>
+      <c r="L271" t="s">
+        <v>282</v>
+      </c>
       <c r="M271" t="s">
-        <v>652</v>
+        <v>535</v>
       </c>
     </row>
     <row r="272" spans="1:13">
@@ -8297,8 +8546,8 @@
       <c r="K272">
         <v>533</v>
       </c>
-      <c r="M272" t="s">
-        <v>653</v>
+      <c r="L272" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="273" spans="1:13">
@@ -8317,8 +8566,11 @@
       <c r="K273">
         <v>515</v>
       </c>
+      <c r="L273" t="s">
+        <v>433</v>
+      </c>
       <c r="M273" t="s">
-        <v>654</v>
+        <v>306</v>
       </c>
     </row>
     <row r="274" spans="1:13">
@@ -8337,8 +8589,11 @@
       <c r="K274">
         <v>510</v>
       </c>
+      <c r="L274" t="s">
+        <v>285</v>
+      </c>
       <c r="M274" t="s">
-        <v>655</v>
+        <v>304</v>
       </c>
     </row>
     <row r="275" spans="1:13">
@@ -8357,8 +8612,8 @@
       <c r="K275">
         <v>464</v>
       </c>
-      <c r="M275" t="s">
-        <v>656</v>
+      <c r="L275" t="s">
+        <v>286</v>
       </c>
     </row>
     <row r="276" spans="1:13">
@@ -8377,8 +8632,8 @@
       <c r="K276">
         <v>480</v>
       </c>
-      <c r="M276" t="s">
-        <v>657</v>
+      <c r="L276" t="s">
+        <v>287</v>
       </c>
     </row>
     <row r="277" spans="1:13">
@@ -8397,8 +8652,11 @@
       <c r="K277">
         <v>535</v>
       </c>
+      <c r="L277" t="s">
+        <v>288</v>
+      </c>
       <c r="M277" t="s">
-        <v>658</v>
+        <v>315</v>
       </c>
     </row>
     <row r="278" spans="1:13">
@@ -8417,8 +8675,8 @@
       <c r="K278">
         <v>536</v>
       </c>
-      <c r="M278" t="s">
-        <v>659</v>
+      <c r="L278" t="s">
+        <v>289</v>
       </c>
     </row>
     <row r="279" spans="1:13">
@@ -8437,8 +8695,8 @@
       <c r="K279">
         <v>516</v>
       </c>
-      <c r="M279" t="s">
-        <v>660</v>
+      <c r="L279" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="280" spans="1:13">
@@ -8460,8 +8718,11 @@
       <c r="K280">
         <v>462</v>
       </c>
+      <c r="L280" t="s">
+        <v>434</v>
+      </c>
       <c r="M280" t="s">
-        <v>661</v>
+        <v>537</v>
       </c>
     </row>
     <row r="281" spans="1:13">
@@ -8483,8 +8744,11 @@
       <c r="K281">
         <v>462</v>
       </c>
+      <c r="L281" t="s">
+        <v>435</v>
+      </c>
       <c r="M281" t="s">
-        <v>662</v>
+        <v>538</v>
       </c>
     </row>
     <row r="282" spans="1:13">
@@ -8506,8 +8770,11 @@
       <c r="K282">
         <v>462</v>
       </c>
+      <c r="L282" t="s">
+        <v>436</v>
+      </c>
       <c r="M282" t="s">
-        <v>663</v>
+        <v>539</v>
       </c>
     </row>
     <row r="283" spans="1:13">
@@ -8526,8 +8793,11 @@
       <c r="K283">
         <v>537</v>
       </c>
+      <c r="L283" t="s">
+        <v>294</v>
+      </c>
       <c r="M283" t="s">
-        <v>664</v>
+        <v>302</v>
       </c>
     </row>
     <row r="284" spans="1:13">
@@ -8546,8 +8816,11 @@
       <c r="K284">
         <v>514</v>
       </c>
+      <c r="L284" t="s">
+        <v>295</v>
+      </c>
       <c r="M284" t="s">
-        <v>665</v>
+        <v>301</v>
       </c>
     </row>
     <row r="285" spans="1:13">
@@ -8563,8 +8836,8 @@
       <c r="K285">
         <v>476</v>
       </c>
-      <c r="M285" t="s">
-        <v>666</v>
+      <c r="L285" t="s">
+        <v>296</v>
       </c>
     </row>
     <row r="286" spans="1:13">
@@ -8580,8 +8853,8 @@
       <c r="K286">
         <v>500</v>
       </c>
-      <c r="M286" t="s">
-        <v>667</v>
+      <c r="L286" t="s">
+        <v>297</v>
       </c>
     </row>
   </sheetData>

</xml_diff>